<commit_message>
Update Export/Import for new version of PackagePassport
</commit_message>
<xml_diff>
--- a/data/Excel/package_passport.xlsx
+++ b/data/Excel/package_passport.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="88">
   <si>
     <t>№</t>
   </si>
@@ -127,9 +127,6 @@
     <t>Отсутствует</t>
   </si>
   <si>
-    <t>Индивидуальный номер упаковки</t>
-  </si>
-  <si>
     <t>Горючесть</t>
   </si>
   <si>
@@ -194,9 +191,6 @@
   </si>
   <si>
     <t>теплоизоляционные материалы неорганические (63), изделия из полимеров (73)</t>
-  </si>
-  <si>
-    <t>Co-60</t>
   </si>
   <si>
     <t>6,44E+04</t>
@@ -333,17 +327,25 @@
   <si>
     <t>на упаковку твердых радиоактивных отходов</t>
   </si>
+  <si>
+    <t>Номер первичной упаковки</t>
+  </si>
+  <si>
+    <t>Тип первичной упаковки</t>
+  </si>
+  <si>
+    <t>Количество и характеристики первичных упаковок</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -396,14 +398,6 @@
     <font>
       <b/>
       <sz val="9"/>
-      <color theme="0"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
       <color theme="0"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
@@ -712,9 +706,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="3" fontId="31" fillId="2" borderId="9"/>
+    <xf numFmtId="3" fontId="30" fillId="2" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -742,53 +736,53 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -797,16 +791,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -814,146 +808,129 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -962,168 +939,191 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1422,7 +1422,8 @@
     <col min="9" max="9" width="9.85546875" style="6" customWidth="1"/>
     <col min="10" max="10" width="10.42578125" style="6" customWidth="1"/>
     <col min="11" max="12" width="11.5703125" style="6" customWidth="1"/>
-    <col min="13" max="14" width="9.7109375" style="6" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" style="6" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="6" customWidth="1"/>
     <col min="15" max="15" width="12" style="6" customWidth="1"/>
     <col min="16" max="16" width="9.7109375" style="6" customWidth="1"/>
     <col min="17" max="17" width="13.42578125" style="6" customWidth="1"/>
@@ -1446,7 +1447,7 @@
       <c r="H1" s="18"/>
       <c r="I1" s="18"/>
       <c r="J1" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K1" s="18"/>
       <c r="L1" s="18"/>
@@ -1457,7 +1458,7 @@
       <c r="Q1" s="18"/>
       <c r="R1" s="18"/>
       <c r="S1" s="53" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="T1" s="53"/>
       <c r="U1" s="53"/>
@@ -1473,7 +1474,7 @@
       <c r="H2" s="18"/>
       <c r="I2" s="18"/>
       <c r="J2" s="19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="K2" s="18"/>
       <c r="L2" s="18"/>
@@ -1493,14 +1494,14 @@
       <c r="F3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="121"/>
-      <c r="H3" s="122"/>
-      <c r="I3" s="122"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
       <c r="J3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="123"/>
-      <c r="L3" s="124"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="135"/>
       <c r="M3" s="25"/>
       <c r="N3" s="26"/>
       <c r="O3" s="22"/>
@@ -1532,7 +1533,7 @@
       <c r="Q4" s="27"/>
       <c r="R4" s="27"/>
       <c r="S4" s="54" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="3" customFormat="1" ht="13.5" x14ac:dyDescent="0.25">
@@ -1545,11 +1546,11 @@
       <c r="G5" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="125"/>
-      <c r="I5" s="126"/>
-      <c r="J5" s="126"/>
-      <c r="K5" s="126"/>
-      <c r="L5" s="126"/>
+      <c r="H5" s="136"/>
+      <c r="I5" s="137"/>
+      <c r="J5" s="137"/>
+      <c r="K5" s="137"/>
+      <c r="L5" s="137"/>
       <c r="M5" s="31"/>
       <c r="N5" s="31"/>
       <c r="O5" s="31"/>
@@ -1568,13 +1569,13 @@
       <c r="E6" s="33"/>
       <c r="F6" s="33"/>
       <c r="G6" s="33"/>
-      <c r="H6" s="113" t="s">
+      <c r="H6" s="138" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="127"/>
-      <c r="J6" s="127"/>
-      <c r="K6" s="127"/>
-      <c r="L6" s="127"/>
+      <c r="I6" s="139"/>
+      <c r="J6" s="139"/>
+      <c r="K6" s="139"/>
+      <c r="L6" s="139"/>
       <c r="M6" s="33"/>
       <c r="N6" s="33"/>
       <c r="O6" s="33"/>
@@ -1587,13 +1588,13 @@
     </row>
     <row r="7" spans="1:21" s="3" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G7" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H7" s="131"/>
-      <c r="I7" s="131"/>
-      <c r="J7" s="131"/>
-      <c r="K7" s="131"/>
-      <c r="L7" s="131"/>
+        <v>65</v>
+      </c>
+      <c r="H7" s="143"/>
+      <c r="I7" s="143"/>
+      <c r="J7" s="143"/>
+      <c r="K7" s="143"/>
+      <c r="L7" s="143"/>
       <c r="S7" s="55">
         <v>4</v>
       </c>
@@ -1606,29 +1607,29 @@
     <row r="9" spans="1:21" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="31"/>
       <c r="B9" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="128"/>
-      <c r="D9" s="129"/>
+        <v>45</v>
+      </c>
+      <c r="C9" s="140"/>
+      <c r="D9" s="141"/>
       <c r="E9" s="31"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="125"/>
-      <c r="H9" s="125"/>
+      <c r="F9" s="136"/>
+      <c r="G9" s="136"/>
+      <c r="H9" s="136"/>
       <c r="I9" s="34"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
-      <c r="L9" s="132"/>
-      <c r="M9" s="132"/>
-      <c r="N9" s="132"/>
-      <c r="O9" s="132"/>
+      <c r="L9" s="144"/>
+      <c r="M9" s="144"/>
+      <c r="N9" s="144"/>
+      <c r="O9" s="144"/>
       <c r="P9" s="34"/>
       <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
       <c r="S9" s="55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="T9" s="55" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U9" s="55" t="str">
         <f>CONCATENATE(T9," куб.м")</f>
@@ -1641,22 +1642,22 @@
       <c r="C10" s="52"/>
       <c r="D10" s="35"/>
       <c r="E10" s="35"/>
-      <c r="F10" s="113" t="s">
+      <c r="F10" s="138" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="113"/>
-      <c r="H10" s="113"/>
+      <c r="G10" s="138"/>
+      <c r="H10" s="138"/>
       <c r="I10" s="35"/>
       <c r="J10" s="35"/>
       <c r="K10" s="35"/>
-      <c r="L10" s="113" t="s">
-        <v>69</v>
-      </c>
-      <c r="M10" s="113"/>
-      <c r="N10" s="113" t="s">
-        <v>68</v>
-      </c>
-      <c r="O10" s="113"/>
+      <c r="L10" s="138" t="s">
+        <v>67</v>
+      </c>
+      <c r="M10" s="138"/>
+      <c r="N10" s="138" t="s">
+        <v>66</v>
+      </c>
+      <c r="O10" s="138"/>
       <c r="P10" s="35"/>
       <c r="Q10" s="35"/>
       <c r="R10" s="35"/>
@@ -1671,12 +1672,12 @@
       <c r="F11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="115"/>
-      <c r="H11" s="115"/>
+      <c r="G11" s="148"/>
+      <c r="H11" s="148"/>
       <c r="I11" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="J11" s="149"/>
+      <c r="J11" s="108"/>
       <c r="K11" s="39"/>
       <c r="L11" s="31"/>
       <c r="M11" s="31"/>
@@ -1696,15 +1697,15 @@
       <c r="F12" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="116"/>
-      <c r="H12" s="116"/>
-      <c r="I12" s="116"/>
+      <c r="G12" s="146"/>
+      <c r="H12" s="146"/>
+      <c r="I12" s="146"/>
       <c r="J12" s="39"/>
       <c r="K12" s="31"/>
-      <c r="L12" s="117"/>
-      <c r="M12" s="117"/>
-      <c r="N12" s="117"/>
-      <c r="O12" s="117"/>
+      <c r="L12" s="147"/>
+      <c r="M12" s="147"/>
+      <c r="N12" s="147"/>
+      <c r="O12" s="147"/>
       <c r="P12" s="37"/>
       <c r="Q12" s="31"/>
       <c r="R12" s="31"/>
@@ -1717,18 +1718,18 @@
       <c r="E13" s="31"/>
       <c r="F13" s="31"/>
       <c r="G13" s="40"/>
-      <c r="H13" s="71" t="s">
+      <c r="H13" s="69" t="s">
         <v>9</v>
       </c>
       <c r="I13" s="45"/>
       <c r="J13" s="39"/>
       <c r="K13" s="31"/>
-      <c r="L13" s="113" t="s">
+      <c r="L13" s="138" t="s">
         <v>10</v>
       </c>
-      <c r="M13" s="113"/>
-      <c r="N13" s="113"/>
-      <c r="O13" s="113"/>
+      <c r="M13" s="138"/>
+      <c r="N13" s="138"/>
+      <c r="O13" s="138"/>
       <c r="P13" s="37"/>
       <c r="Q13" s="41"/>
       <c r="R13" s="28"/>
@@ -1742,14 +1743,14 @@
       <c r="F14" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="117"/>
-      <c r="H14" s="117"/>
-      <c r="I14" s="117"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="117"/>
-      <c r="L14" s="117"/>
+      <c r="G14" s="147"/>
+      <c r="H14" s="147"/>
+      <c r="I14" s="147"/>
+      <c r="J14" s="147"/>
+      <c r="K14" s="147"/>
+      <c r="L14" s="147"/>
       <c r="M14" s="56" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N14" s="150"/>
       <c r="O14" s="150"/>
@@ -1766,14 +1767,14 @@
       <c r="F15" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="133"/>
-      <c r="H15" s="133"/>
-      <c r="I15" s="133"/>
-      <c r="J15" s="133"/>
-      <c r="K15" s="133"/>
-      <c r="L15" s="133"/>
+      <c r="G15" s="149"/>
+      <c r="H15" s="149"/>
+      <c r="I15" s="149"/>
+      <c r="J15" s="149"/>
+      <c r="K15" s="149"/>
+      <c r="L15" s="149"/>
       <c r="M15" s="56" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N15" s="151"/>
       <c r="O15" s="151"/>
@@ -1790,17 +1791,17 @@
       <c r="F16" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="125"/>
-      <c r="H16" s="125"/>
-      <c r="I16" s="125"/>
+      <c r="G16" s="136"/>
+      <c r="H16" s="136"/>
+      <c r="I16" s="136"/>
       <c r="J16" s="39"/>
       <c r="K16" s="31"/>
       <c r="L16" s="31"/>
       <c r="M16" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="N16" s="114"/>
-      <c r="O16" s="114"/>
+      <c r="N16" s="145"/>
+      <c r="O16" s="145"/>
       <c r="P16" s="31"/>
       <c r="Q16" s="45"/>
       <c r="R16" s="31"/>
@@ -1814,11 +1815,11 @@
       <c r="F17" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="152"/>
-      <c r="H17" s="153" t="s">
-        <v>83</v>
-      </c>
-      <c r="I17" s="154"/>
+      <c r="G17" s="109"/>
+      <c r="H17" s="110" t="s">
+        <v>81</v>
+      </c>
+      <c r="I17" s="111"/>
       <c r="J17" s="45"/>
       <c r="K17" s="43"/>
       <c r="L17" s="43"/>
@@ -1838,7 +1839,7 @@
       <c r="F18" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="160"/>
+      <c r="G18" s="113"/>
       <c r="H18" s="45"/>
       <c r="I18" s="45"/>
       <c r="J18" s="45"/>
@@ -1847,8 +1848,8 @@
       <c r="M18" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="N18" s="130"/>
-      <c r="O18" s="130"/>
+      <c r="N18" s="142"/>
+      <c r="O18" s="142"/>
       <c r="P18" s="43"/>
       <c r="Q18" s="45"/>
       <c r="R18" s="37"/>
@@ -1872,478 +1873,492 @@
       <c r="P19" s="46"/>
       <c r="Q19" s="46"/>
       <c r="R19" s="46"/>
-      <c r="S19" s="68" t="s">
+      <c r="S19" s="66" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" s="7" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="96" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="123" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="123"/>
+      <c r="D20" s="123"/>
+      <c r="E20" s="123"/>
+      <c r="F20" s="123"/>
+      <c r="G20" s="123"/>
+      <c r="H20" s="123"/>
+      <c r="I20" s="123"/>
+      <c r="J20" s="123"/>
+      <c r="K20" s="123"/>
+      <c r="L20" s="123"/>
+      <c r="M20" s="123"/>
+      <c r="N20" s="123"/>
+      <c r="O20" s="123"/>
+      <c r="P20" s="123"/>
+      <c r="S20" s="68"/>
+      <c r="T20" s="105"/>
+      <c r="U20" s="105"/>
+      <c r="V20" s="105"/>
+    </row>
+    <row r="21" spans="1:23" s="7" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="119" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="120"/>
+      <c r="C21" s="121"/>
+      <c r="D21" s="119" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="120"/>
+      <c r="F21" s="120"/>
+      <c r="G21" s="121"/>
+      <c r="H21" s="117" t="s">
+        <v>78</v>
+      </c>
+      <c r="I21" s="118"/>
+      <c r="J21" s="117" t="s">
+        <v>79</v>
+      </c>
+      <c r="K21" s="118"/>
+      <c r="L21" s="117" t="s">
+        <v>64</v>
+      </c>
+      <c r="M21" s="118"/>
+      <c r="N21" s="117" t="s">
+        <v>60</v>
+      </c>
+      <c r="O21" s="118"/>
+      <c r="P21" s="126" t="s">
+        <v>68</v>
+      </c>
+      <c r="S21" s="68">
+        <v>17</v>
+      </c>
+      <c r="T21" s="98"/>
+      <c r="U21" s="98"/>
+      <c r="V21" s="105"/>
+    </row>
+    <row r="22" spans="1:23" s="7" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="92" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="92" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="92" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="106" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="106" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="106" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="106" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="92" t="s">
+        <v>62</v>
+      </c>
+      <c r="I22" s="92" t="s">
+        <v>28</v>
+      </c>
+      <c r="J22" s="92" t="s">
+        <v>62</v>
+      </c>
+      <c r="K22" s="92" t="s">
+        <v>28</v>
+      </c>
+      <c r="L22" s="92">
+        <v>0.1</v>
+      </c>
+      <c r="M22" s="92">
+        <v>1</v>
+      </c>
+      <c r="N22" s="92" t="s">
+        <v>73</v>
+      </c>
+      <c r="O22" s="92" t="s">
+        <v>74</v>
+      </c>
+      <c r="P22" s="127"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="102" t="s">
+        <v>31</v>
+      </c>
+      <c r="T22" s="103">
+        <v>1500</v>
+      </c>
+      <c r="U22" s="104"/>
+      <c r="V22" s="101"/>
+      <c r="W22" s="8"/>
+    </row>
+    <row r="23" spans="1:23" s="8" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="93">
+        <v>1</v>
+      </c>
+      <c r="B23" s="93">
+        <v>2</v>
+      </c>
+      <c r="C23" s="93">
+        <v>3</v>
+      </c>
+      <c r="D23" s="93">
+        <v>4</v>
+      </c>
+      <c r="E23" s="93">
+        <v>5</v>
+      </c>
+      <c r="F23" s="93">
+        <v>6</v>
+      </c>
+      <c r="G23" s="93">
+        <v>7</v>
+      </c>
+      <c r="H23" s="93">
+        <v>8</v>
+      </c>
+      <c r="I23" s="93">
+        <v>9</v>
+      </c>
+      <c r="J23" s="93">
+        <v>10</v>
+      </c>
+      <c r="K23" s="93">
+        <v>11</v>
+      </c>
+      <c r="L23" s="93">
+        <v>12</v>
+      </c>
+      <c r="M23" s="93">
+        <v>13</v>
+      </c>
+      <c r="N23" s="94">
+        <v>14</v>
+      </c>
+      <c r="O23" s="101">
+        <v>15</v>
+      </c>
+      <c r="P23" s="101">
+        <v>16</v>
+      </c>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" s="99"/>
+      <c r="T23" s="100"/>
+      <c r="U23" s="98"/>
+      <c r="V23" s="97"/>
+      <c r="W23" s="9"/>
+    </row>
+    <row r="24" spans="1:23" s="9" customFormat="1" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="81"/>
+      <c r="B24" s="68"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
+      <c r="K24" s="68"/>
+      <c r="L24" s="68"/>
+      <c r="M24" s="68"/>
+      <c r="N24" s="81"/>
+      <c r="O24" s="81"/>
+      <c r="P24" s="97"/>
+      <c r="Q24" s="76"/>
+      <c r="R24" s="62"/>
+      <c r="S24" s="77"/>
+      <c r="T24" s="78"/>
+      <c r="U24" s="72"/>
+      <c r="V24" s="11"/>
+      <c r="W24" s="11"/>
+    </row>
+    <row r="25" spans="1:23" s="11" customFormat="1" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="62"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="74"/>
+      <c r="I25" s="62"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="62"/>
+      <c r="L25" s="62"/>
+      <c r="M25" s="62"/>
+      <c r="N25" s="62"/>
+      <c r="O25" s="75"/>
+      <c r="Q25" s="82"/>
+      <c r="R25" s="82"/>
+      <c r="S25" s="79"/>
+      <c r="T25" s="79"/>
+      <c r="U25" s="79"/>
+      <c r="V25" s="79"/>
+      <c r="W25" s="79"/>
+    </row>
+    <row r="26" spans="1:23" s="10" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="155" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="123" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" spans="1:23" s="7" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="103" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" s="143" t="s">
+      <c r="C26" s="123"/>
+      <c r="D26" s="123"/>
+      <c r="E26" s="123"/>
+      <c r="F26" s="123"/>
+      <c r="G26" s="123"/>
+      <c r="H26" s="123"/>
+      <c r="I26" s="123"/>
+      <c r="J26" s="123"/>
+      <c r="K26" s="123"/>
+      <c r="L26" s="123"/>
+      <c r="M26" s="123"/>
+      <c r="N26" s="123"/>
+      <c r="O26" s="123"/>
+      <c r="P26" s="123"/>
+      <c r="Q26" s="123"/>
+      <c r="R26" s="123"/>
+      <c r="S26" s="123"/>
+      <c r="T26" s="123"/>
+      <c r="U26" s="123"/>
+      <c r="V26" s="123"/>
+      <c r="W26" s="123"/>
+    </row>
+    <row r="27" spans="1:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="122" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="156" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="122" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="122" t="s">
+        <v>69</v>
+      </c>
+      <c r="E27" s="122" t="s">
+        <v>71</v>
+      </c>
+      <c r="F27" s="122" t="s">
+        <v>72</v>
+      </c>
+      <c r="G27" s="122" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="156" t="s">
+        <v>87</v>
+      </c>
+      <c r="I27" s="156"/>
+      <c r="J27" s="156"/>
+      <c r="K27" s="122" t="s">
+        <v>33</v>
+      </c>
+      <c r="L27" s="122" t="s">
+        <v>34</v>
+      </c>
+      <c r="M27" s="122" t="s">
+        <v>77</v>
+      </c>
+      <c r="N27" s="122"/>
+      <c r="O27" s="122"/>
+      <c r="P27" s="122"/>
+      <c r="Q27" s="122"/>
+      <c r="R27" s="122" t="s">
+        <v>35</v>
+      </c>
+      <c r="S27" s="106"/>
+      <c r="T27" s="153"/>
+      <c r="U27" s="153"/>
+      <c r="V27" s="153"/>
+      <c r="W27" s="156" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="122"/>
+      <c r="B28" s="156"/>
+      <c r="C28" s="122"/>
+      <c r="D28" s="122"/>
+      <c r="E28" s="122"/>
+      <c r="F28" s="122"/>
+      <c r="G28" s="122"/>
+      <c r="H28" s="153" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28" s="106" t="s">
+        <v>79</v>
+      </c>
+      <c r="J28" s="106" t="s">
+        <v>30</v>
+      </c>
+      <c r="K28" s="122"/>
+      <c r="L28" s="122"/>
+      <c r="M28" s="106" t="s">
+        <v>36</v>
+      </c>
+      <c r="N28" s="106" t="s">
+        <v>37</v>
+      </c>
+      <c r="O28" s="106" t="s">
+        <v>38</v>
+      </c>
+      <c r="P28" s="106" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q28" s="106" t="s">
+        <v>39</v>
+      </c>
+      <c r="R28" s="122"/>
+      <c r="S28" s="152">
+        <v>15</v>
+      </c>
+      <c r="T28" s="157"/>
+      <c r="U28" s="157"/>
+      <c r="V28" s="153"/>
+      <c r="W28" s="156"/>
+    </row>
+    <row r="29" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="95">
+        <v>1</v>
+      </c>
+      <c r="B29" s="107">
+        <v>2</v>
+      </c>
+      <c r="C29" s="95">
+        <v>3</v>
+      </c>
+      <c r="D29" s="95">
+        <v>4</v>
+      </c>
+      <c r="E29" s="106">
+        <v>5</v>
+      </c>
+      <c r="F29" s="106">
+        <v>6</v>
+      </c>
+      <c r="G29" s="106">
+        <v>7</v>
+      </c>
+      <c r="H29" s="95">
+        <v>8</v>
+      </c>
+      <c r="I29" s="95">
+        <v>9</v>
+      </c>
+      <c r="J29" s="95">
+        <v>10</v>
+      </c>
+      <c r="K29" s="95">
+        <v>11</v>
+      </c>
+      <c r="L29" s="95">
+        <v>12</v>
+      </c>
+      <c r="M29" s="95">
+        <v>13</v>
+      </c>
+      <c r="N29" s="95">
+        <v>14</v>
+      </c>
+      <c r="O29" s="95">
+        <v>15</v>
+      </c>
+      <c r="P29" s="95">
+        <v>16</v>
+      </c>
+      <c r="Q29" s="95">
+        <v>17</v>
+      </c>
+      <c r="R29" s="95">
         <v>18</v>
       </c>
-      <c r="C20" s="144"/>
-      <c r="D20" s="144"/>
-      <c r="E20" s="144"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="144"/>
-      <c r="I20" s="144"/>
-      <c r="J20" s="144"/>
-      <c r="K20" s="144"/>
-      <c r="L20" s="144"/>
-      <c r="M20" s="144"/>
-      <c r="N20" s="144"/>
-      <c r="O20" s="144"/>
-      <c r="P20" s="144"/>
-      <c r="Q20" s="144"/>
-      <c r="R20" s="144"/>
-      <c r="S20" s="144"/>
-      <c r="T20" s="144"/>
-      <c r="U20" s="144"/>
-      <c r="V20" s="144"/>
-      <c r="W20" s="145"/>
-    </row>
-    <row r="21" spans="1:23" s="7" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="134" t="s">
+      <c r="S29" s="154"/>
+      <c r="T29" s="158" t="s">
+        <v>54</v>
+      </c>
+      <c r="U29" s="159" t="s">
+        <v>55</v>
+      </c>
+      <c r="V29" s="160"/>
+      <c r="W29" s="160">
         <v>19</v>
       </c>
-      <c r="B21" s="135"/>
-      <c r="C21" s="135"/>
-      <c r="D21" s="135"/>
-      <c r="E21" s="135"/>
-      <c r="F21" s="136"/>
-      <c r="G21" s="134" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" s="135"/>
-      <c r="I21" s="135"/>
-      <c r="J21" s="136"/>
-      <c r="K21" s="141" t="s">
-        <v>80</v>
-      </c>
-      <c r="L21" s="142"/>
-      <c r="M21" s="141" t="s">
-        <v>81</v>
-      </c>
-      <c r="N21" s="142"/>
-      <c r="O21" s="141" t="s">
-        <v>66</v>
-      </c>
-      <c r="P21" s="142"/>
-      <c r="Q21" s="141" t="s">
-        <v>62</v>
-      </c>
-      <c r="R21" s="142"/>
-      <c r="S21" s="70"/>
-      <c r="T21" s="112"/>
-      <c r="U21" s="112"/>
-      <c r="V21" s="112"/>
-      <c r="W21" s="139" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:23" s="7" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="99" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="99" t="s">
-        <v>73</v>
-      </c>
-      <c r="C22" s="99" t="s">
-        <v>74</v>
-      </c>
-      <c r="D22" s="99" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="99" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" s="99" t="s">
-        <v>23</v>
-      </c>
-      <c r="G22" s="99" t="s">
-        <v>24</v>
-      </c>
-      <c r="H22" s="99" t="s">
-        <v>25</v>
-      </c>
-      <c r="I22" s="99" t="s">
-        <v>26</v>
-      </c>
-      <c r="J22" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K22" s="99" t="s">
-        <v>64</v>
-      </c>
-      <c r="L22" s="99" t="s">
-        <v>28</v>
-      </c>
-      <c r="M22" s="99" t="s">
-        <v>64</v>
-      </c>
-      <c r="N22" s="99" t="s">
-        <v>28</v>
-      </c>
-      <c r="O22" s="99">
-        <v>0.1</v>
-      </c>
-      <c r="P22" s="99">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="99" t="s">
-        <v>75</v>
-      </c>
-      <c r="R22" s="99" t="s">
-        <v>76</v>
-      </c>
-      <c r="S22" s="70">
-        <v>17</v>
-      </c>
-      <c r="T22" s="105"/>
-      <c r="U22" s="105"/>
-      <c r="V22" s="112"/>
-      <c r="W22" s="140"/>
-    </row>
-    <row r="23" spans="1:23" s="8" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="100">
-        <v>1</v>
-      </c>
-      <c r="B23" s="100">
-        <v>2</v>
-      </c>
-      <c r="C23" s="100">
-        <v>3</v>
-      </c>
-      <c r="D23" s="100">
-        <v>4</v>
-      </c>
-      <c r="E23" s="100">
-        <v>5</v>
-      </c>
-      <c r="F23" s="100">
-        <v>6</v>
-      </c>
-      <c r="G23" s="100">
-        <v>7</v>
-      </c>
-      <c r="H23" s="100">
-        <v>8</v>
-      </c>
-      <c r="I23" s="100">
-        <v>9</v>
-      </c>
-      <c r="J23" s="100">
-        <v>10</v>
-      </c>
-      <c r="K23" s="100">
-        <v>11</v>
-      </c>
-      <c r="L23" s="100">
-        <v>12</v>
-      </c>
-      <c r="M23" s="100">
-        <v>13</v>
-      </c>
-      <c r="N23" s="100">
-        <v>14</v>
-      </c>
-      <c r="O23" s="100">
-        <v>15</v>
-      </c>
-      <c r="P23" s="100">
-        <v>16</v>
-      </c>
-      <c r="Q23" s="101">
-        <v>17</v>
-      </c>
-      <c r="R23" s="108">
-        <v>18</v>
-      </c>
-      <c r="S23" s="109" t="s">
-        <v>31</v>
-      </c>
-      <c r="T23" s="110">
-        <v>1500</v>
-      </c>
-      <c r="U23" s="111"/>
-      <c r="V23" s="108"/>
-      <c r="W23" s="108">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" s="9" customFormat="1" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="85"/>
-      <c r="B24" s="85"/>
-      <c r="C24" s="85"/>
-      <c r="D24" s="70"/>
-      <c r="E24" s="70"/>
-      <c r="F24" s="70"/>
-      <c r="G24" s="70"/>
-      <c r="H24" s="70"/>
-      <c r="I24" s="70"/>
-      <c r="J24" s="70"/>
-      <c r="K24" s="70"/>
-      <c r="L24" s="70"/>
-      <c r="M24" s="70"/>
-      <c r="N24" s="70"/>
-      <c r="O24" s="70"/>
-      <c r="P24" s="70"/>
-      <c r="Q24" s="85"/>
-      <c r="R24" s="85"/>
-      <c r="S24" s="106"/>
-      <c r="T24" s="107"/>
-      <c r="U24" s="105"/>
-      <c r="V24" s="104"/>
-      <c r="W24" s="104"/>
-    </row>
-    <row r="25" spans="1:23" s="11" customFormat="1" ht="13.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="63"/>
-      <c r="B25" s="63"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="77"/>
-      <c r="I25" s="63"/>
-      <c r="J25" s="63"/>
-      <c r="K25" s="63"/>
-      <c r="L25" s="63"/>
-      <c r="M25" s="63"/>
-      <c r="N25" s="63"/>
-      <c r="O25" s="78"/>
-      <c r="P25" s="78"/>
-      <c r="Q25" s="79"/>
-      <c r="R25" s="63"/>
-      <c r="S25" s="80"/>
-      <c r="T25" s="81"/>
-      <c r="U25" s="75"/>
-    </row>
-    <row r="26" spans="1:23" s="10" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="103" t="s">
-        <v>51</v>
-      </c>
-      <c r="B26" s="148" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="148"/>
-      <c r="D26" s="148"/>
-      <c r="E26" s="148"/>
-      <c r="F26" s="148"/>
-      <c r="G26" s="148"/>
-      <c r="H26" s="148"/>
-      <c r="I26" s="148"/>
-      <c r="J26" s="148"/>
-      <c r="K26" s="148"/>
-      <c r="L26" s="148"/>
-      <c r="M26" s="148"/>
-      <c r="N26" s="148"/>
-      <c r="O26" s="148"/>
-      <c r="P26" s="86"/>
-      <c r="Q26" s="86"/>
-      <c r="R26" s="86"/>
-      <c r="S26" s="82"/>
-      <c r="T26" s="82"/>
-      <c r="U26" s="82"/>
-      <c r="V26" s="82"/>
-      <c r="W26" s="82"/>
-    </row>
-    <row r="27" spans="1:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="146" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="146" t="s">
-        <v>72</v>
-      </c>
-      <c r="C27" s="146" t="s">
-        <v>71</v>
-      </c>
-      <c r="D27" s="147" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="146" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="146" t="s">
-        <v>30</v>
-      </c>
-      <c r="G27" s="146" t="s">
-        <v>34</v>
-      </c>
-      <c r="H27" s="146" t="s">
-        <v>35</v>
-      </c>
-      <c r="I27" s="146" t="s">
-        <v>79</v>
-      </c>
-      <c r="J27" s="146"/>
-      <c r="K27" s="146"/>
-      <c r="L27" s="146"/>
-      <c r="M27" s="146"/>
-      <c r="N27" s="146" t="s">
-        <v>36</v>
-      </c>
-      <c r="O27" s="146" t="s">
-        <v>78</v>
-      </c>
-      <c r="P27" s="87"/>
-      <c r="Q27" s="74"/>
-      <c r="R27" s="88"/>
-      <c r="S27" s="84"/>
-      <c r="T27" s="84"/>
-      <c r="U27" s="84"/>
-      <c r="V27" s="84"/>
-      <c r="W27" s="84"/>
-    </row>
-    <row r="28" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="146"/>
-      <c r="B28" s="146"/>
-      <c r="C28" s="146"/>
-      <c r="D28" s="147"/>
-      <c r="E28" s="146"/>
-      <c r="F28" s="146"/>
-      <c r="G28" s="146"/>
-      <c r="H28" s="146"/>
-      <c r="I28" s="99" t="s">
-        <v>37</v>
-      </c>
-      <c r="J28" s="99" t="s">
-        <v>38</v>
-      </c>
-      <c r="K28" s="99" t="s">
-        <v>39</v>
-      </c>
-      <c r="L28" s="99" t="s">
-        <v>77</v>
-      </c>
-      <c r="M28" s="99" t="s">
-        <v>40</v>
-      </c>
-      <c r="N28" s="146"/>
-      <c r="O28" s="146"/>
-      <c r="P28" s="87"/>
-      <c r="Q28" s="74"/>
-      <c r="R28" s="74"/>
-    </row>
-    <row r="29" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="102">
-        <v>1</v>
-      </c>
-      <c r="B29" s="102">
-        <v>2</v>
-      </c>
-      <c r="C29" s="102">
-        <v>3</v>
-      </c>
-      <c r="D29" s="102">
-        <v>4</v>
-      </c>
-      <c r="E29" s="102">
-        <v>5</v>
-      </c>
-      <c r="F29" s="102">
-        <v>6</v>
-      </c>
-      <c r="G29" s="102">
-        <v>7</v>
-      </c>
-      <c r="H29" s="102">
-        <v>8</v>
-      </c>
-      <c r="I29" s="102">
-        <v>9</v>
-      </c>
-      <c r="J29" s="102">
-        <v>10</v>
-      </c>
-      <c r="K29" s="102">
-        <v>11</v>
-      </c>
-      <c r="L29" s="102">
-        <v>12</v>
-      </c>
-      <c r="M29" s="102">
-        <v>13</v>
-      </c>
-      <c r="N29" s="102">
-        <v>14</v>
-      </c>
-      <c r="O29" s="102">
-        <v>15</v>
-      </c>
-      <c r="P29" s="65"/>
-      <c r="Q29" s="89"/>
-      <c r="R29" s="76"/>
-      <c r="S29" s="58" t="s">
-        <v>45</v>
-      </c>
-      <c r="T29" s="60"/>
-      <c r="U29" s="60"/>
     </row>
     <row r="30" spans="1:23" s="5" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="95"/>
-      <c r="B30" s="95"/>
-      <c r="C30" s="95"/>
-      <c r="D30" s="95"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="96"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
-      <c r="J30" s="96"/>
-      <c r="K30" s="96"/>
-      <c r="L30" s="98"/>
-      <c r="M30" s="98"/>
-      <c r="N30" s="97"/>
-      <c r="O30" s="97"/>
-      <c r="P30" s="64"/>
-      <c r="Q30" s="89"/>
-      <c r="R30" s="76"/>
-      <c r="S30" s="59" t="s">
+      <c r="A30" s="88"/>
+      <c r="B30" s="161"/>
+      <c r="C30" s="88"/>
+      <c r="D30" s="88"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="88"/>
+      <c r="I30" s="89"/>
+      <c r="J30" s="89"/>
+      <c r="K30" s="89"/>
+      <c r="L30" s="89"/>
+      <c r="M30" s="89"/>
+      <c r="N30" s="89"/>
+      <c r="O30" s="89"/>
+      <c r="P30" s="91"/>
+      <c r="Q30" s="91"/>
+      <c r="R30" s="90"/>
+      <c r="S30" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="T30" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="U30" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="T30" s="59" t="s">
-        <v>56</v>
-      </c>
-      <c r="U30" s="61" t="s">
-        <v>57</v>
-      </c>
+      <c r="V30" s="161"/>
+      <c r="W30" s="161"/>
     </row>
     <row r="31" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="76"/>
-      <c r="B31" s="76"/>
-      <c r="C31" s="90"/>
-      <c r="D31" s="90"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="73"/>
-      <c r="H31" s="73"/>
-      <c r="I31" s="73"/>
-      <c r="J31" s="73"/>
-      <c r="K31" s="73"/>
-      <c r="L31" s="63"/>
-      <c r="M31" s="91"/>
-      <c r="N31" s="69"/>
-      <c r="O31" s="72"/>
-      <c r="P31" s="64"/>
-      <c r="Q31" s="89"/>
-      <c r="R31" s="76"/>
-      <c r="S31" s="59" t="s">
-        <v>58</v>
-      </c>
-      <c r="T31" s="59" t="s">
-        <v>59</v>
-      </c>
-      <c r="U31" s="61" t="s">
-        <v>57</v>
+      <c r="A31" s="73"/>
+      <c r="B31" s="73"/>
+      <c r="C31" s="83"/>
+      <c r="D31" s="83"/>
+      <c r="E31" s="71"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="71"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="71"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="62"/>
+      <c r="M31" s="84"/>
+      <c r="N31" s="67"/>
+      <c r="O31" s="70"/>
+      <c r="P31" s="63"/>
+      <c r="Q31" s="49"/>
+      <c r="R31" s="49"/>
+      <c r="S31" s="58">
+        <v>0</v>
+      </c>
+      <c r="T31" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U31" s="60" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="49"/>
       <c r="C32" s="49"/>
@@ -2362,46 +2377,46 @@
       <c r="P32" s="49"/>
       <c r="Q32" s="49"/>
       <c r="R32" s="49"/>
-      <c r="S32" s="59">
+      <c r="S32" s="58">
         <v>0</v>
       </c>
-      <c r="T32" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U32" s="61" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" s="5" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="156"/>
-      <c r="B33" s="156"/>
-      <c r="C33" s="156"/>
-      <c r="D33" s="156"/>
-      <c r="E33" s="156"/>
-      <c r="F33" s="156"/>
-      <c r="G33" s="155"/>
-      <c r="H33" s="155"/>
-      <c r="I33" s="155"/>
-      <c r="J33" s="155"/>
-      <c r="K33" s="155"/>
-      <c r="L33" s="155"/>
-      <c r="M33" s="155"/>
-      <c r="N33" s="155"/>
-      <c r="O33" s="155"/>
+      <c r="T32" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U32" s="60" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" s="5" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="128"/>
+      <c r="B33" s="128"/>
+      <c r="C33" s="128"/>
+      <c r="D33" s="128"/>
+      <c r="E33" s="128"/>
+      <c r="F33" s="128"/>
+      <c r="G33" s="112"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+      <c r="J33" s="112"/>
+      <c r="K33" s="112"/>
+      <c r="L33" s="112"/>
+      <c r="M33" s="112"/>
+      <c r="N33" s="112"/>
+      <c r="O33" s="112"/>
       <c r="P33" s="49"/>
-      <c r="Q33" s="49"/>
-      <c r="R33" s="49"/>
-      <c r="S33" s="59">
+      <c r="Q33" s="50"/>
+      <c r="R33" s="50"/>
+      <c r="S33" s="58">
         <v>0</v>
       </c>
-      <c r="T33" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U33" s="61" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T33" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U33" s="60" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15"/>
       <c r="B34" s="50"/>
       <c r="C34" s="50"/>
@@ -2418,236 +2433,281 @@
       <c r="N34" s="50"/>
       <c r="O34" s="50"/>
       <c r="P34" s="50"/>
-      <c r="Q34" s="50"/>
-      <c r="R34" s="50"/>
-      <c r="S34" s="59">
+      <c r="Q34" s="125"/>
+      <c r="R34" s="125"/>
+      <c r="S34" s="58">
         <v>0</v>
       </c>
-      <c r="T34" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U34" s="61" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T34" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U34" s="59"/>
+    </row>
+    <row r="35" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="31"/>
       <c r="B35" s="51"/>
       <c r="D35" s="51"/>
       <c r="E35" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="F35" s="157"/>
-      <c r="G35" s="157"/>
-      <c r="H35" s="157"/>
-      <c r="I35" s="67"/>
-      <c r="J35" s="158"/>
-      <c r="K35" s="158"/>
-      <c r="L35" s="158"/>
-      <c r="M35" s="158"/>
-      <c r="N35" s="158"/>
-      <c r="O35" s="158"/>
+        <v>40</v>
+      </c>
+      <c r="F35" s="129"/>
+      <c r="G35" s="129"/>
+      <c r="H35" s="129"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="116"/>
+      <c r="K35" s="116"/>
+      <c r="L35" s="116"/>
+      <c r="M35" s="116"/>
+      <c r="N35" s="116"/>
+      <c r="O35" s="116"/>
       <c r="P35" s="43"/>
-      <c r="Q35" s="138"/>
-      <c r="R35" s="138"/>
-      <c r="S35" s="59">
-        <v>0</v>
-      </c>
-      <c r="T35" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U35" s="60"/>
-    </row>
-    <row r="36" spans="1:21" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q35" s="125"/>
+      <c r="R35" s="125"/>
+      <c r="S35" s="58"/>
+      <c r="T35" s="58"/>
+      <c r="U35" s="59"/>
+      <c r="V35" s="3"/>
+      <c r="W35" s="3"/>
+    </row>
+    <row r="36" spans="1:23" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="43"/>
       <c r="B36" s="51"/>
       <c r="C36" s="5"/>
       <c r="D36" s="43"/>
       <c r="E36" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="F36" s="137"/>
-      <c r="G36" s="137"/>
-      <c r="H36" s="137"/>
+        <v>43</v>
+      </c>
+      <c r="F36" s="124"/>
+      <c r="G36" s="124"/>
+      <c r="H36" s="124"/>
       <c r="I36" s="43"/>
-      <c r="J36" s="159"/>
-      <c r="K36" s="159"/>
-      <c r="L36" s="159"/>
-      <c r="M36" s="159"/>
-      <c r="N36" s="159"/>
-      <c r="O36" s="159"/>
+      <c r="J36" s="115"/>
+      <c r="K36" s="115"/>
+      <c r="L36" s="115"/>
+      <c r="M36" s="115"/>
+      <c r="N36" s="115"/>
+      <c r="O36" s="115"/>
       <c r="P36" s="43"/>
-      <c r="Q36" s="138"/>
-      <c r="R36" s="138"/>
-      <c r="S36" s="59"/>
-      <c r="T36" s="59"/>
-      <c r="U36" s="60"/>
-    </row>
-    <row r="37" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="118"/>
-      <c r="B37" s="118"/>
-      <c r="C37" s="118"/>
-      <c r="D37" s="118"/>
+      <c r="Q36" s="131" t="s">
+        <v>42</v>
+      </c>
+      <c r="R36" s="131"/>
+      <c r="S36" s="58"/>
+      <c r="T36" s="58"/>
+      <c r="U36" s="59"/>
+      <c r="V36" s="5"/>
+      <c r="W36" s="5"/>
+    </row>
+    <row r="37" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="130"/>
+      <c r="B37" s="130"/>
+      <c r="C37" s="130"/>
+      <c r="D37" s="130"/>
       <c r="E37" s="4"/>
-      <c r="F37" s="119" t="s">
-        <v>42</v>
-      </c>
-      <c r="G37" s="119"/>
-      <c r="H37" s="119"/>
+      <c r="F37" s="131" t="s">
+        <v>41</v>
+      </c>
+      <c r="G37" s="131"/>
+      <c r="H37" s="131"/>
       <c r="I37" s="33"/>
-      <c r="J37" s="120" t="s">
-        <v>84</v>
-      </c>
-      <c r="K37" s="120"/>
-      <c r="L37" s="120"/>
-      <c r="M37" s="120" t="s">
-        <v>85</v>
-      </c>
-      <c r="N37" s="120"/>
-      <c r="O37" s="120"/>
+      <c r="J37" s="114" t="s">
+        <v>82</v>
+      </c>
+      <c r="K37" s="114"/>
+      <c r="L37" s="114"/>
+      <c r="M37" s="114" t="s">
+        <v>83</v>
+      </c>
+      <c r="N37" s="114"/>
+      <c r="O37" s="114"/>
       <c r="P37" s="33"/>
-      <c r="Q37" s="119" t="s">
-        <v>43</v>
-      </c>
-      <c r="R37" s="119"/>
-      <c r="S37" s="59"/>
-      <c r="T37" s="59"/>
-      <c r="U37" s="60"/>
-    </row>
-    <row r="38" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="90"/>
-      <c r="B38" s="90"/>
-      <c r="C38" s="90"/>
-      <c r="D38" s="90"/>
-      <c r="E38" s="73"/>
-      <c r="F38" s="73"/>
-      <c r="G38" s="73"/>
-      <c r="H38" s="73"/>
-      <c r="I38" s="73"/>
-      <c r="J38" s="73"/>
-      <c r="K38" s="73"/>
-      <c r="L38" s="64"/>
-      <c r="M38" s="66"/>
-      <c r="N38" s="92"/>
-      <c r="O38" s="83"/>
-      <c r="P38" s="93"/>
-      <c r="Q38" s="94"/>
-      <c r="R38" s="76"/>
-      <c r="S38" s="59"/>
-      <c r="T38" s="59"/>
-      <c r="U38" s="60"/>
-    </row>
-    <row r="39" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="S39" s="59"/>
-      <c r="T39" s="59"/>
-      <c r="U39" s="60" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:21" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:21" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:21" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:21" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:21" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="62"/>
-      <c r="B48" s="62"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="62"/>
-      <c r="L48" s="62"/>
-      <c r="M48" s="62"/>
-      <c r="N48" s="62"/>
-      <c r="O48" s="62"/>
-      <c r="P48" s="62"/>
-      <c r="Q48" s="62"/>
-      <c r="R48" s="62"/>
+      <c r="Q37" s="87"/>
+      <c r="R37" s="73"/>
+      <c r="S37" s="58"/>
+      <c r="T37" s="58"/>
+      <c r="U37" s="59"/>
+    </row>
+    <row r="38" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="83"/>
+      <c r="B38" s="83"/>
+      <c r="C38" s="83"/>
+      <c r="D38" s="83"/>
+      <c r="E38" s="71"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="71"/>
+      <c r="H38" s="71"/>
+      <c r="I38" s="71"/>
+      <c r="J38" s="71"/>
+      <c r="K38" s="71"/>
+      <c r="L38" s="63"/>
+      <c r="M38" s="64"/>
+      <c r="N38" s="85"/>
+      <c r="O38" s="80"/>
+      <c r="P38" s="86"/>
+      <c r="S38" s="58"/>
+      <c r="T38" s="58"/>
+      <c r="U38" s="59" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q39" s="13"/>
+      <c r="R39" s="13"/>
+      <c r="S39" s="13"/>
+      <c r="T39" s="13"/>
+      <c r="U39" s="13"/>
+      <c r="V39" s="13"/>
+      <c r="W39" s="13"/>
+    </row>
+    <row r="40" spans="1:23" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:23" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q41" s="15"/>
+      <c r="R41" s="15"/>
+      <c r="S41" s="15"/>
+      <c r="T41" s="15"/>
+      <c r="U41" s="15"/>
+      <c r="V41" s="15"/>
+      <c r="W41" s="15"/>
+    </row>
+    <row r="42" spans="1:23" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
+      <c r="S42" s="5"/>
+      <c r="T42" s="5"/>
+      <c r="U42" s="5"/>
+      <c r="V42" s="5"/>
+      <c r="W42" s="5"/>
+    </row>
+    <row r="43" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q43" s="4"/>
+      <c r="R43" s="4"/>
+      <c r="S43" s="4"/>
+      <c r="T43" s="4"/>
+      <c r="U43" s="4"/>
+      <c r="V43" s="4"/>
+      <c r="W43" s="4"/>
+    </row>
+    <row r="44" spans="1:23" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q44" s="16"/>
+      <c r="R44" s="16"/>
+      <c r="S44" s="16"/>
+      <c r="T44" s="16"/>
+      <c r="U44" s="16"/>
+      <c r="V44" s="16"/>
+      <c r="W44" s="16"/>
+    </row>
+    <row r="45" spans="1:23" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q45" s="5"/>
+      <c r="R45" s="5"/>
+      <c r="S45" s="5"/>
+      <c r="T45" s="5"/>
+      <c r="U45" s="5"/>
+      <c r="V45" s="5"/>
+      <c r="W45" s="5"/>
+    </row>
+    <row r="46" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="4"/>
+      <c r="T46" s="4"/>
+      <c r="U46" s="4"/>
+      <c r="V46" s="4"/>
+      <c r="W46" s="4"/>
+    </row>
+    <row r="47" spans="1:23" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q47" s="61"/>
+      <c r="R47" s="61"/>
+      <c r="S47" s="6"/>
+      <c r="T47" s="6"/>
+      <c r="U47" s="6"/>
+      <c r="V47" s="6"/>
+      <c r="W47" s="6"/>
+    </row>
+    <row r="48" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A48" s="61"/>
+      <c r="B48" s="61"/>
+      <c r="C48" s="61"/>
+      <c r="D48" s="61"/>
+      <c r="E48" s="61"/>
+      <c r="F48" s="61"/>
+      <c r="G48" s="61"/>
+      <c r="H48" s="61"/>
+      <c r="I48" s="61"/>
+      <c r="J48" s="61"/>
+      <c r="K48" s="61"/>
+      <c r="L48" s="61"/>
+      <c r="M48" s="61"/>
+      <c r="N48" s="61"/>
+      <c r="O48" s="61"/>
+      <c r="P48" s="61"/>
+      <c r="Q48" s="61"/>
+      <c r="R48" s="61"/>
     </row>
     <row r="49" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="62"/>
-      <c r="B49" s="62"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="62"/>
-      <c r="L49" s="62"/>
-      <c r="M49" s="62"/>
-      <c r="N49" s="62"/>
-      <c r="O49" s="62"/>
-      <c r="P49" s="62"/>
-      <c r="Q49" s="62"/>
-      <c r="R49" s="62"/>
+      <c r="A49" s="61"/>
+      <c r="B49" s="61"/>
+      <c r="C49" s="61"/>
+      <c r="D49" s="61"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="61"/>
+      <c r="G49" s="61"/>
+      <c r="H49" s="61"/>
+      <c r="I49" s="61"/>
+      <c r="J49" s="61"/>
+      <c r="K49" s="61"/>
+      <c r="L49" s="61"/>
+      <c r="M49" s="61"/>
+      <c r="N49" s="61"/>
+      <c r="O49" s="61"/>
+      <c r="P49" s="61"/>
+      <c r="Q49" s="61"/>
+      <c r="R49" s="61"/>
     </row>
     <row r="50" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="62"/>
-      <c r="B50" s="62"/>
-      <c r="C50" s="62"/>
-      <c r="D50" s="62"/>
-      <c r="E50" s="62"/>
-      <c r="F50" s="62"/>
-      <c r="G50" s="62"/>
-      <c r="H50" s="62"/>
-      <c r="I50" s="62"/>
-      <c r="J50" s="62"/>
-      <c r="K50" s="62"/>
-      <c r="L50" s="62"/>
-      <c r="M50" s="62"/>
-      <c r="N50" s="62"/>
-      <c r="O50" s="62"/>
-      <c r="P50" s="62"/>
-      <c r="Q50" s="62"/>
-      <c r="R50" s="62"/>
+      <c r="A50" s="61"/>
+      <c r="B50" s="61"/>
+      <c r="C50" s="61"/>
+      <c r="D50" s="61"/>
+      <c r="E50" s="61"/>
+      <c r="F50" s="61"/>
+      <c r="G50" s="61"/>
+      <c r="H50" s="61"/>
+      <c r="I50" s="61"/>
+      <c r="J50" s="61"/>
+      <c r="K50" s="61"/>
+      <c r="L50" s="61"/>
+      <c r="M50" s="61"/>
+      <c r="N50" s="61"/>
+      <c r="O50" s="61"/>
+      <c r="P50" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
-    <mergeCell ref="J37:L37"/>
-    <mergeCell ref="M37:O37"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J35:L35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="M36:O36"/>
-    <mergeCell ref="B20:W20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="A27:A28"/>
+  <mergeCells count="59">
+    <mergeCell ref="B20:P20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:G21"/>
     <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="E27:E28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B26:O26"/>
     <mergeCell ref="F27:F28"/>
     <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:M27"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="W21:W22"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="M27:Q27"/>
+    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G14:L14"/>
+    <mergeCell ref="G15:L15"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="L12:O12"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="F37:H37"/>
-    <mergeCell ref="Q37:R37"/>
+    <mergeCell ref="Q36:R36"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="H5:L5"/>
@@ -2661,16 +2721,27 @@
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="F10:H10"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G14:L14"/>
-    <mergeCell ref="G15:L15"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="P21:P22"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="R27:R28"/>
+    <mergeCell ref="W27:W28"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="J37:L37"/>
+    <mergeCell ref="M37:O37"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="J35:L35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M36:O36"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.31496062992125984" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.11811023622047245"/>
   <pageSetup paperSize="9" scale="83" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Reapply "Merge branch '1.3.0.4-Passports-branch' into 1.3.0.7"
This reverts commit 2bcd1c3a9b67bc8a2beb02765e57114451fd00a1.
</commit_message>
<xml_diff>
--- a/data/Excel/package_passport.xlsx
+++ b/data/Excel/package_passport.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="88">
   <si>
     <t>№</t>
   </si>
@@ -127,9 +127,6 @@
     <t>Отсутствует</t>
   </si>
   <si>
-    <t>Индивидуальный номер упаковки</t>
-  </si>
-  <si>
     <t>Горючесть</t>
   </si>
   <si>
@@ -194,9 +191,6 @@
   </si>
   <si>
     <t>теплоизоляционные материалы неорганические (63), изделия из полимеров (73)</t>
-  </si>
-  <si>
-    <t>Co-60</t>
   </si>
   <si>
     <t>6,44E+04</t>
@@ -333,17 +327,25 @@
   <si>
     <t>на упаковку твердых радиоактивных отходов</t>
   </si>
+  <si>
+    <t>Номер первичной упаковки</t>
+  </si>
+  <si>
+    <t>Тип первичной упаковки</t>
+  </si>
+  <si>
+    <t>Количество и характеристики первичных упаковок</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.000E+00"/>
   </numFmts>
-  <fonts count="32" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -396,14 +398,6 @@
     <font>
       <b/>
       <sz val="9"/>
-      <color theme="0"/>
-      <name val="Arial Narrow"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
       <color theme="0"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
@@ -712,9 +706,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="3" fontId="31" fillId="2" borderId="9"/>
+    <xf numFmtId="3" fontId="30" fillId="2" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="163">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -742,53 +736,53 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -797,16 +791,16 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -814,146 +808,129 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="11" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -962,168 +939,191 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="9" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="23" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="25" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1422,7 +1422,8 @@
     <col min="9" max="9" width="9.85546875" style="6" customWidth="1"/>
     <col min="10" max="10" width="10.42578125" style="6" customWidth="1"/>
     <col min="11" max="12" width="11.5703125" style="6" customWidth="1"/>
-    <col min="13" max="14" width="9.7109375" style="6" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" style="6" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" style="6" customWidth="1"/>
     <col min="15" max="15" width="12" style="6" customWidth="1"/>
     <col min="16" max="16" width="9.7109375" style="6" customWidth="1"/>
     <col min="17" max="17" width="13.42578125" style="6" customWidth="1"/>
@@ -1446,7 +1447,7 @@
       <c r="H1" s="18"/>
       <c r="I1" s="18"/>
       <c r="J1" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K1" s="18"/>
       <c r="L1" s="18"/>
@@ -1457,7 +1458,7 @@
       <c r="Q1" s="18"/>
       <c r="R1" s="18"/>
       <c r="S1" s="53" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="T1" s="53"/>
       <c r="U1" s="53"/>
@@ -1473,7 +1474,7 @@
       <c r="H2" s="18"/>
       <c r="I2" s="18"/>
       <c r="J2" s="19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="K2" s="18"/>
       <c r="L2" s="18"/>
@@ -1493,14 +1494,14 @@
       <c r="F3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="121"/>
-      <c r="H3" s="122"/>
-      <c r="I3" s="122"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
       <c r="J3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="123"/>
-      <c r="L3" s="124"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="135"/>
       <c r="M3" s="25"/>
       <c r="N3" s="26"/>
       <c r="O3" s="22"/>
@@ -1532,7 +1533,7 @@
       <c r="Q4" s="27"/>
       <c r="R4" s="27"/>
       <c r="S4" s="54" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="3" customFormat="1" ht="13.5" x14ac:dyDescent="0.25">
@@ -1545,11 +1546,11 @@
       <c r="G5" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="125"/>
-      <c r="I5" s="126"/>
-      <c r="J5" s="126"/>
-      <c r="K5" s="126"/>
-      <c r="L5" s="126"/>
+      <c r="H5" s="136"/>
+      <c r="I5" s="137"/>
+      <c r="J5" s="137"/>
+      <c r="K5" s="137"/>
+      <c r="L5" s="137"/>
       <c r="M5" s="31"/>
       <c r="N5" s="31"/>
       <c r="O5" s="31"/>
@@ -1568,13 +1569,13 @@
       <c r="E6" s="33"/>
       <c r="F6" s="33"/>
       <c r="G6" s="33"/>
-      <c r="H6" s="113" t="s">
+      <c r="H6" s="138" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="127"/>
-      <c r="J6" s="127"/>
-      <c r="K6" s="127"/>
-      <c r="L6" s="127"/>
+      <c r="I6" s="139"/>
+      <c r="J6" s="139"/>
+      <c r="K6" s="139"/>
+      <c r="L6" s="139"/>
       <c r="M6" s="33"/>
       <c r="N6" s="33"/>
       <c r="O6" s="33"/>
@@ -1587,13 +1588,13 @@
     </row>
     <row r="7" spans="1:21" s="3" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G7" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="H7" s="131"/>
-      <c r="I7" s="131"/>
-      <c r="J7" s="131"/>
-      <c r="K7" s="131"/>
-      <c r="L7" s="131"/>
+        <v>65</v>
+      </c>
+      <c r="H7" s="143"/>
+      <c r="I7" s="143"/>
+      <c r="J7" s="143"/>
+      <c r="K7" s="143"/>
+      <c r="L7" s="143"/>
       <c r="S7" s="55">
         <v>4</v>
       </c>
@@ -1606,29 +1607,29 @@
     <row r="9" spans="1:21" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="31"/>
       <c r="B9" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="128"/>
-      <c r="D9" s="129"/>
+        <v>45</v>
+      </c>
+      <c r="C9" s="140"/>
+      <c r="D9" s="141"/>
       <c r="E9" s="31"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="125"/>
-      <c r="H9" s="125"/>
+      <c r="F9" s="136"/>
+      <c r="G9" s="136"/>
+      <c r="H9" s="136"/>
       <c r="I9" s="34"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
-      <c r="L9" s="132"/>
-      <c r="M9" s="132"/>
-      <c r="N9" s="132"/>
-      <c r="O9" s="132"/>
+      <c r="L9" s="144"/>
+      <c r="M9" s="144"/>
+      <c r="N9" s="144"/>
+      <c r="O9" s="144"/>
       <c r="P9" s="34"/>
       <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
       <c r="S9" s="55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="T9" s="55" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="U9" s="55" t="str">
         <f>CONCATENATE(T9," куб.м")</f>
@@ -1641,22 +1642,22 @@
       <c r="C10" s="52"/>
       <c r="D10" s="35"/>
       <c r="E10" s="35"/>
-      <c r="F10" s="113" t="s">
+      <c r="F10" s="138" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="113"/>
-      <c r="H10" s="113"/>
+      <c r="G10" s="138"/>
+      <c r="H10" s="138"/>
       <c r="I10" s="35"/>
       <c r="J10" s="35"/>
       <c r="K10" s="35"/>
-      <c r="L10" s="113" t="s">
-        <v>69</v>
-      </c>
-      <c r="M10" s="113"/>
-      <c r="N10" s="113" t="s">
-        <v>68</v>
-      </c>
-      <c r="O10" s="113"/>
+      <c r="L10" s="138" t="s">
+        <v>67</v>
+      </c>
+      <c r="M10" s="138"/>
+      <c r="N10" s="138" t="s">
+        <v>66</v>
+      </c>
+      <c r="O10" s="138"/>
       <c r="P10" s="35"/>
       <c r="Q10" s="35"/>
       <c r="R10" s="35"/>
@@ -1671,12 +1672,12 @@
       <c r="F11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="115"/>
-      <c r="H11" s="115"/>
+      <c r="G11" s="148"/>
+      <c r="H11" s="148"/>
       <c r="I11" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="J11" s="149"/>
+      <c r="J11" s="108"/>
       <c r="K11" s="39"/>
       <c r="L11" s="31"/>
       <c r="M11" s="31"/>
@@ -1696,15 +1697,15 @@
       <c r="F12" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="116"/>
-      <c r="H12" s="116"/>
-      <c r="I12" s="116"/>
+      <c r="G12" s="146"/>
+      <c r="H12" s="146"/>
+      <c r="I12" s="146"/>
       <c r="J12" s="39"/>
       <c r="K12" s="31"/>
-      <c r="L12" s="117"/>
-      <c r="M12" s="117"/>
-      <c r="N12" s="117"/>
-      <c r="O12" s="117"/>
+      <c r="L12" s="147"/>
+      <c r="M12" s="147"/>
+      <c r="N12" s="147"/>
+      <c r="O12" s="147"/>
       <c r="P12" s="37"/>
       <c r="Q12" s="31"/>
       <c r="R12" s="31"/>
@@ -1717,18 +1718,18 @@
       <c r="E13" s="31"/>
       <c r="F13" s="31"/>
       <c r="G13" s="40"/>
-      <c r="H13" s="71" t="s">
+      <c r="H13" s="69" t="s">
         <v>9</v>
       </c>
       <c r="I13" s="45"/>
       <c r="J13" s="39"/>
       <c r="K13" s="31"/>
-      <c r="L13" s="113" t="s">
+      <c r="L13" s="138" t="s">
         <v>10</v>
       </c>
-      <c r="M13" s="113"/>
-      <c r="N13" s="113"/>
-      <c r="O13" s="113"/>
+      <c r="M13" s="138"/>
+      <c r="N13" s="138"/>
+      <c r="O13" s="138"/>
       <c r="P13" s="37"/>
       <c r="Q13" s="41"/>
       <c r="R13" s="28"/>
@@ -1742,14 +1743,14 @@
       <c r="F14" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="117"/>
-      <c r="H14" s="117"/>
-      <c r="I14" s="117"/>
-      <c r="J14" s="117"/>
-      <c r="K14" s="117"/>
-      <c r="L14" s="117"/>
+      <c r="G14" s="147"/>
+      <c r="H14" s="147"/>
+      <c r="I14" s="147"/>
+      <c r="J14" s="147"/>
+      <c r="K14" s="147"/>
+      <c r="L14" s="147"/>
       <c r="M14" s="56" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N14" s="150"/>
       <c r="O14" s="150"/>
@@ -1766,14 +1767,14 @@
       <c r="F15" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="133"/>
-      <c r="H15" s="133"/>
-      <c r="I15" s="133"/>
-      <c r="J15" s="133"/>
-      <c r="K15" s="133"/>
-      <c r="L15" s="133"/>
+      <c r="G15" s="149"/>
+      <c r="H15" s="149"/>
+      <c r="I15" s="149"/>
+      <c r="J15" s="149"/>
+      <c r="K15" s="149"/>
+      <c r="L15" s="149"/>
       <c r="M15" s="56" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="N15" s="151"/>
       <c r="O15" s="151"/>
@@ -1790,17 +1791,17 @@
       <c r="F16" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="125"/>
-      <c r="H16" s="125"/>
-      <c r="I16" s="125"/>
+      <c r="G16" s="136"/>
+      <c r="H16" s="136"/>
+      <c r="I16" s="136"/>
       <c r="J16" s="39"/>
       <c r="K16" s="31"/>
       <c r="L16" s="31"/>
       <c r="M16" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="N16" s="114"/>
-      <c r="O16" s="114"/>
+      <c r="N16" s="145"/>
+      <c r="O16" s="145"/>
       <c r="P16" s="31"/>
       <c r="Q16" s="45"/>
       <c r="R16" s="31"/>
@@ -1814,11 +1815,11 @@
       <c r="F17" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="152"/>
-      <c r="H17" s="153" t="s">
-        <v>83</v>
-      </c>
-      <c r="I17" s="154"/>
+      <c r="G17" s="109"/>
+      <c r="H17" s="110" t="s">
+        <v>81</v>
+      </c>
+      <c r="I17" s="111"/>
       <c r="J17" s="45"/>
       <c r="K17" s="43"/>
       <c r="L17" s="43"/>
@@ -1838,7 +1839,7 @@
       <c r="F18" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="160"/>
+      <c r="G18" s="113"/>
       <c r="H18" s="45"/>
       <c r="I18" s="45"/>
       <c r="J18" s="45"/>
@@ -1847,8 +1848,8 @@
       <c r="M18" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="N18" s="130"/>
-      <c r="O18" s="130"/>
+      <c r="N18" s="142"/>
+      <c r="O18" s="142"/>
       <c r="P18" s="43"/>
       <c r="Q18" s="45"/>
       <c r="R18" s="37"/>
@@ -1872,478 +1873,492 @@
       <c r="P19" s="46"/>
       <c r="Q19" s="46"/>
       <c r="R19" s="46"/>
-      <c r="S19" s="68" t="s">
+      <c r="S19" s="66" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" s="7" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="96" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="123" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="123"/>
+      <c r="D20" s="123"/>
+      <c r="E20" s="123"/>
+      <c r="F20" s="123"/>
+      <c r="G20" s="123"/>
+      <c r="H20" s="123"/>
+      <c r="I20" s="123"/>
+      <c r="J20" s="123"/>
+      <c r="K20" s="123"/>
+      <c r="L20" s="123"/>
+      <c r="M20" s="123"/>
+      <c r="N20" s="123"/>
+      <c r="O20" s="123"/>
+      <c r="P20" s="123"/>
+      <c r="S20" s="68"/>
+      <c r="T20" s="105"/>
+      <c r="U20" s="105"/>
+      <c r="V20" s="105"/>
+    </row>
+    <row r="21" spans="1:23" s="7" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="119" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="120"/>
+      <c r="C21" s="121"/>
+      <c r="D21" s="119" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="120"/>
+      <c r="F21" s="120"/>
+      <c r="G21" s="121"/>
+      <c r="H21" s="117" t="s">
+        <v>78</v>
+      </c>
+      <c r="I21" s="118"/>
+      <c r="J21" s="117" t="s">
+        <v>79</v>
+      </c>
+      <c r="K21" s="118"/>
+      <c r="L21" s="117" t="s">
+        <v>64</v>
+      </c>
+      <c r="M21" s="118"/>
+      <c r="N21" s="117" t="s">
+        <v>60</v>
+      </c>
+      <c r="O21" s="118"/>
+      <c r="P21" s="126" t="s">
+        <v>68</v>
+      </c>
+      <c r="S21" s="68">
+        <v>17</v>
+      </c>
+      <c r="T21" s="98"/>
+      <c r="U21" s="98"/>
+      <c r="V21" s="105"/>
+    </row>
+    <row r="22" spans="1:23" s="7" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="92" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="92" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="92" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="106" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" s="106" t="s">
+        <v>25</v>
+      </c>
+      <c r="F22" s="106" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="106" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="92" t="s">
+        <v>62</v>
+      </c>
+      <c r="I22" s="92" t="s">
+        <v>28</v>
+      </c>
+      <c r="J22" s="92" t="s">
+        <v>62</v>
+      </c>
+      <c r="K22" s="92" t="s">
+        <v>28</v>
+      </c>
+      <c r="L22" s="92">
+        <v>0.1</v>
+      </c>
+      <c r="M22" s="92">
+        <v>1</v>
+      </c>
+      <c r="N22" s="92" t="s">
+        <v>73</v>
+      </c>
+      <c r="O22" s="92" t="s">
+        <v>74</v>
+      </c>
+      <c r="P22" s="127"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="102" t="s">
+        <v>31</v>
+      </c>
+      <c r="T22" s="103">
+        <v>1500</v>
+      </c>
+      <c r="U22" s="104"/>
+      <c r="V22" s="101"/>
+      <c r="W22" s="8"/>
+    </row>
+    <row r="23" spans="1:23" s="8" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="93">
+        <v>1</v>
+      </c>
+      <c r="B23" s="93">
+        <v>2</v>
+      </c>
+      <c r="C23" s="93">
+        <v>3</v>
+      </c>
+      <c r="D23" s="93">
+        <v>4</v>
+      </c>
+      <c r="E23" s="93">
+        <v>5</v>
+      </c>
+      <c r="F23" s="93">
+        <v>6</v>
+      </c>
+      <c r="G23" s="93">
+        <v>7</v>
+      </c>
+      <c r="H23" s="93">
+        <v>8</v>
+      </c>
+      <c r="I23" s="93">
+        <v>9</v>
+      </c>
+      <c r="J23" s="93">
+        <v>10</v>
+      </c>
+      <c r="K23" s="93">
+        <v>11</v>
+      </c>
+      <c r="L23" s="93">
+        <v>12</v>
+      </c>
+      <c r="M23" s="93">
+        <v>13</v>
+      </c>
+      <c r="N23" s="94">
+        <v>14</v>
+      </c>
+      <c r="O23" s="101">
+        <v>15</v>
+      </c>
+      <c r="P23" s="101">
+        <v>16</v>
+      </c>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" s="99"/>
+      <c r="T23" s="100"/>
+      <c r="U23" s="98"/>
+      <c r="V23" s="97"/>
+      <c r="W23" s="9"/>
+    </row>
+    <row r="24" spans="1:23" s="9" customFormat="1" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="81"/>
+      <c r="B24" s="68"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="68"/>
+      <c r="E24" s="68"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="68"/>
+      <c r="K24" s="68"/>
+      <c r="L24" s="68"/>
+      <c r="M24" s="68"/>
+      <c r="N24" s="81"/>
+      <c r="O24" s="81"/>
+      <c r="P24" s="97"/>
+      <c r="Q24" s="76"/>
+      <c r="R24" s="62"/>
+      <c r="S24" s="77"/>
+      <c r="T24" s="78"/>
+      <c r="U24" s="72"/>
+      <c r="V24" s="11"/>
+      <c r="W24" s="11"/>
+    </row>
+    <row r="25" spans="1:23" s="11" customFormat="1" ht="13.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="62"/>
+      <c r="B25" s="62"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="62"/>
+      <c r="E25" s="62"/>
+      <c r="F25" s="62"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="74"/>
+      <c r="I25" s="62"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="62"/>
+      <c r="L25" s="62"/>
+      <c r="M25" s="62"/>
+      <c r="N25" s="62"/>
+      <c r="O25" s="75"/>
+      <c r="Q25" s="82"/>
+      <c r="R25" s="82"/>
+      <c r="S25" s="79"/>
+      <c r="T25" s="79"/>
+      <c r="U25" s="79"/>
+      <c r="V25" s="79"/>
+      <c r="W25" s="79"/>
+    </row>
+    <row r="26" spans="1:23" s="10" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="155" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="123" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" spans="1:23" s="7" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="103" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" s="143" t="s">
+      <c r="C26" s="123"/>
+      <c r="D26" s="123"/>
+      <c r="E26" s="123"/>
+      <c r="F26" s="123"/>
+      <c r="G26" s="123"/>
+      <c r="H26" s="123"/>
+      <c r="I26" s="123"/>
+      <c r="J26" s="123"/>
+      <c r="K26" s="123"/>
+      <c r="L26" s="123"/>
+      <c r="M26" s="123"/>
+      <c r="N26" s="123"/>
+      <c r="O26" s="123"/>
+      <c r="P26" s="123"/>
+      <c r="Q26" s="123"/>
+      <c r="R26" s="123"/>
+      <c r="S26" s="123"/>
+      <c r="T26" s="123"/>
+      <c r="U26" s="123"/>
+      <c r="V26" s="123"/>
+      <c r="W26" s="123"/>
+    </row>
+    <row r="27" spans="1:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="122" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" s="156" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" s="122" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="122" t="s">
+        <v>69</v>
+      </c>
+      <c r="E27" s="122" t="s">
+        <v>71</v>
+      </c>
+      <c r="F27" s="122" t="s">
+        <v>72</v>
+      </c>
+      <c r="G27" s="122" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="156" t="s">
+        <v>87</v>
+      </c>
+      <c r="I27" s="156"/>
+      <c r="J27" s="156"/>
+      <c r="K27" s="122" t="s">
+        <v>33</v>
+      </c>
+      <c r="L27" s="122" t="s">
+        <v>34</v>
+      </c>
+      <c r="M27" s="122" t="s">
+        <v>77</v>
+      </c>
+      <c r="N27" s="122"/>
+      <c r="O27" s="122"/>
+      <c r="P27" s="122"/>
+      <c r="Q27" s="122"/>
+      <c r="R27" s="122" t="s">
+        <v>35</v>
+      </c>
+      <c r="S27" s="106"/>
+      <c r="T27" s="153"/>
+      <c r="U27" s="153"/>
+      <c r="V27" s="153"/>
+      <c r="W27" s="156" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="122"/>
+      <c r="B28" s="156"/>
+      <c r="C28" s="122"/>
+      <c r="D28" s="122"/>
+      <c r="E28" s="122"/>
+      <c r="F28" s="122"/>
+      <c r="G28" s="122"/>
+      <c r="H28" s="153" t="s">
+        <v>29</v>
+      </c>
+      <c r="I28" s="106" t="s">
+        <v>79</v>
+      </c>
+      <c r="J28" s="106" t="s">
+        <v>30</v>
+      </c>
+      <c r="K28" s="122"/>
+      <c r="L28" s="122"/>
+      <c r="M28" s="106" t="s">
+        <v>36</v>
+      </c>
+      <c r="N28" s="106" t="s">
+        <v>37</v>
+      </c>
+      <c r="O28" s="106" t="s">
+        <v>38</v>
+      </c>
+      <c r="P28" s="106" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q28" s="106" t="s">
+        <v>39</v>
+      </c>
+      <c r="R28" s="122"/>
+      <c r="S28" s="152">
+        <v>15</v>
+      </c>
+      <c r="T28" s="157"/>
+      <c r="U28" s="157"/>
+      <c r="V28" s="153"/>
+      <c r="W28" s="156"/>
+    </row>
+    <row r="29" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="95">
+        <v>1</v>
+      </c>
+      <c r="B29" s="107">
+        <v>2</v>
+      </c>
+      <c r="C29" s="95">
+        <v>3</v>
+      </c>
+      <c r="D29" s="95">
+        <v>4</v>
+      </c>
+      <c r="E29" s="106">
+        <v>5</v>
+      </c>
+      <c r="F29" s="106">
+        <v>6</v>
+      </c>
+      <c r="G29" s="106">
+        <v>7</v>
+      </c>
+      <c r="H29" s="95">
+        <v>8</v>
+      </c>
+      <c r="I29" s="95">
+        <v>9</v>
+      </c>
+      <c r="J29" s="95">
+        <v>10</v>
+      </c>
+      <c r="K29" s="95">
+        <v>11</v>
+      </c>
+      <c r="L29" s="95">
+        <v>12</v>
+      </c>
+      <c r="M29" s="95">
+        <v>13</v>
+      </c>
+      <c r="N29" s="95">
+        <v>14</v>
+      </c>
+      <c r="O29" s="95">
+        <v>15</v>
+      </c>
+      <c r="P29" s="95">
+        <v>16</v>
+      </c>
+      <c r="Q29" s="95">
+        <v>17</v>
+      </c>
+      <c r="R29" s="95">
         <v>18</v>
       </c>
-      <c r="C20" s="144"/>
-      <c r="D20" s="144"/>
-      <c r="E20" s="144"/>
-      <c r="F20" s="144"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="144"/>
-      <c r="I20" s="144"/>
-      <c r="J20" s="144"/>
-      <c r="K20" s="144"/>
-      <c r="L20" s="144"/>
-      <c r="M20" s="144"/>
-      <c r="N20" s="144"/>
-      <c r="O20" s="144"/>
-      <c r="P20" s="144"/>
-      <c r="Q20" s="144"/>
-      <c r="R20" s="144"/>
-      <c r="S20" s="144"/>
-      <c r="T20" s="144"/>
-      <c r="U20" s="144"/>
-      <c r="V20" s="144"/>
-      <c r="W20" s="145"/>
-    </row>
-    <row r="21" spans="1:23" s="7" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="134" t="s">
+      <c r="S29" s="154"/>
+      <c r="T29" s="158" t="s">
+        <v>54</v>
+      </c>
+      <c r="U29" s="159" t="s">
+        <v>55</v>
+      </c>
+      <c r="V29" s="160"/>
+      <c r="W29" s="160">
         <v>19</v>
       </c>
-      <c r="B21" s="135"/>
-      <c r="C21" s="135"/>
-      <c r="D21" s="135"/>
-      <c r="E21" s="135"/>
-      <c r="F21" s="136"/>
-      <c r="G21" s="134" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" s="135"/>
-      <c r="I21" s="135"/>
-      <c r="J21" s="136"/>
-      <c r="K21" s="141" t="s">
-        <v>80</v>
-      </c>
-      <c r="L21" s="142"/>
-      <c r="M21" s="141" t="s">
-        <v>81</v>
-      </c>
-      <c r="N21" s="142"/>
-      <c r="O21" s="141" t="s">
-        <v>66</v>
-      </c>
-      <c r="P21" s="142"/>
-      <c r="Q21" s="141" t="s">
-        <v>62</v>
-      </c>
-      <c r="R21" s="142"/>
-      <c r="S21" s="70"/>
-      <c r="T21" s="112"/>
-      <c r="U21" s="112"/>
-      <c r="V21" s="112"/>
-      <c r="W21" s="139" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:23" s="7" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="99" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="99" t="s">
-        <v>73</v>
-      </c>
-      <c r="C22" s="99" t="s">
-        <v>74</v>
-      </c>
-      <c r="D22" s="99" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="99" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" s="99" t="s">
-        <v>23</v>
-      </c>
-      <c r="G22" s="99" t="s">
-        <v>24</v>
-      </c>
-      <c r="H22" s="99" t="s">
-        <v>25</v>
-      </c>
-      <c r="I22" s="99" t="s">
-        <v>26</v>
-      </c>
-      <c r="J22" s="99" t="s">
-        <v>27</v>
-      </c>
-      <c r="K22" s="99" t="s">
-        <v>64</v>
-      </c>
-      <c r="L22" s="99" t="s">
-        <v>28</v>
-      </c>
-      <c r="M22" s="99" t="s">
-        <v>64</v>
-      </c>
-      <c r="N22" s="99" t="s">
-        <v>28</v>
-      </c>
-      <c r="O22" s="99">
-        <v>0.1</v>
-      </c>
-      <c r="P22" s="99">
-        <v>1</v>
-      </c>
-      <c r="Q22" s="99" t="s">
-        <v>75</v>
-      </c>
-      <c r="R22" s="99" t="s">
-        <v>76</v>
-      </c>
-      <c r="S22" s="70">
-        <v>17</v>
-      </c>
-      <c r="T22" s="105"/>
-      <c r="U22" s="105"/>
-      <c r="V22" s="112"/>
-      <c r="W22" s="140"/>
-    </row>
-    <row r="23" spans="1:23" s="8" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="100">
-        <v>1</v>
-      </c>
-      <c r="B23" s="100">
-        <v>2</v>
-      </c>
-      <c r="C23" s="100">
-        <v>3</v>
-      </c>
-      <c r="D23" s="100">
-        <v>4</v>
-      </c>
-      <c r="E23" s="100">
-        <v>5</v>
-      </c>
-      <c r="F23" s="100">
-        <v>6</v>
-      </c>
-      <c r="G23" s="100">
-        <v>7</v>
-      </c>
-      <c r="H23" s="100">
-        <v>8</v>
-      </c>
-      <c r="I23" s="100">
-        <v>9</v>
-      </c>
-      <c r="J23" s="100">
-        <v>10</v>
-      </c>
-      <c r="K23" s="100">
-        <v>11</v>
-      </c>
-      <c r="L23" s="100">
-        <v>12</v>
-      </c>
-      <c r="M23" s="100">
-        <v>13</v>
-      </c>
-      <c r="N23" s="100">
-        <v>14</v>
-      </c>
-      <c r="O23" s="100">
-        <v>15</v>
-      </c>
-      <c r="P23" s="100">
-        <v>16</v>
-      </c>
-      <c r="Q23" s="101">
-        <v>17</v>
-      </c>
-      <c r="R23" s="108">
-        <v>18</v>
-      </c>
-      <c r="S23" s="109" t="s">
-        <v>31</v>
-      </c>
-      <c r="T23" s="110">
-        <v>1500</v>
-      </c>
-      <c r="U23" s="111"/>
-      <c r="V23" s="108"/>
-      <c r="W23" s="108">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" s="9" customFormat="1" ht="83.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="85"/>
-      <c r="B24" s="85"/>
-      <c r="C24" s="85"/>
-      <c r="D24" s="70"/>
-      <c r="E24" s="70"/>
-      <c r="F24" s="70"/>
-      <c r="G24" s="70"/>
-      <c r="H24" s="70"/>
-      <c r="I24" s="70"/>
-      <c r="J24" s="70"/>
-      <c r="K24" s="70"/>
-      <c r="L24" s="70"/>
-      <c r="M24" s="70"/>
-      <c r="N24" s="70"/>
-      <c r="O24" s="70"/>
-      <c r="P24" s="70"/>
-      <c r="Q24" s="85"/>
-      <c r="R24" s="85"/>
-      <c r="S24" s="106"/>
-      <c r="T24" s="107"/>
-      <c r="U24" s="105"/>
-      <c r="V24" s="104"/>
-      <c r="W24" s="104"/>
-    </row>
-    <row r="25" spans="1:23" s="11" customFormat="1" ht="13.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="63"/>
-      <c r="B25" s="63"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="63"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="77"/>
-      <c r="I25" s="63"/>
-      <c r="J25" s="63"/>
-      <c r="K25" s="63"/>
-      <c r="L25" s="63"/>
-      <c r="M25" s="63"/>
-      <c r="N25" s="63"/>
-      <c r="O25" s="78"/>
-      <c r="P25" s="78"/>
-      <c r="Q25" s="79"/>
-      <c r="R25" s="63"/>
-      <c r="S25" s="80"/>
-      <c r="T25" s="81"/>
-      <c r="U25" s="75"/>
-    </row>
-    <row r="26" spans="1:23" s="10" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="103" t="s">
-        <v>51</v>
-      </c>
-      <c r="B26" s="148" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="148"/>
-      <c r="D26" s="148"/>
-      <c r="E26" s="148"/>
-      <c r="F26" s="148"/>
-      <c r="G26" s="148"/>
-      <c r="H26" s="148"/>
-      <c r="I26" s="148"/>
-      <c r="J26" s="148"/>
-      <c r="K26" s="148"/>
-      <c r="L26" s="148"/>
-      <c r="M26" s="148"/>
-      <c r="N26" s="148"/>
-      <c r="O26" s="148"/>
-      <c r="P26" s="86"/>
-      <c r="Q26" s="86"/>
-      <c r="R26" s="86"/>
-      <c r="S26" s="82"/>
-      <c r="T26" s="82"/>
-      <c r="U26" s="82"/>
-      <c r="V26" s="82"/>
-      <c r="W26" s="82"/>
-    </row>
-    <row r="27" spans="1:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="146" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="146" t="s">
-        <v>72</v>
-      </c>
-      <c r="C27" s="146" t="s">
-        <v>71</v>
-      </c>
-      <c r="D27" s="147" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="146" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="146" t="s">
-        <v>30</v>
-      </c>
-      <c r="G27" s="146" t="s">
-        <v>34</v>
-      </c>
-      <c r="H27" s="146" t="s">
-        <v>35</v>
-      </c>
-      <c r="I27" s="146" t="s">
-        <v>79</v>
-      </c>
-      <c r="J27" s="146"/>
-      <c r="K27" s="146"/>
-      <c r="L27" s="146"/>
-      <c r="M27" s="146"/>
-      <c r="N27" s="146" t="s">
-        <v>36</v>
-      </c>
-      <c r="O27" s="146" t="s">
-        <v>78</v>
-      </c>
-      <c r="P27" s="87"/>
-      <c r="Q27" s="74"/>
-      <c r="R27" s="88"/>
-      <c r="S27" s="84"/>
-      <c r="T27" s="84"/>
-      <c r="U27" s="84"/>
-      <c r="V27" s="84"/>
-      <c r="W27" s="84"/>
-    </row>
-    <row r="28" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="146"/>
-      <c r="B28" s="146"/>
-      <c r="C28" s="146"/>
-      <c r="D28" s="147"/>
-      <c r="E28" s="146"/>
-      <c r="F28" s="146"/>
-      <c r="G28" s="146"/>
-      <c r="H28" s="146"/>
-      <c r="I28" s="99" t="s">
-        <v>37</v>
-      </c>
-      <c r="J28" s="99" t="s">
-        <v>38</v>
-      </c>
-      <c r="K28" s="99" t="s">
-        <v>39</v>
-      </c>
-      <c r="L28" s="99" t="s">
-        <v>77</v>
-      </c>
-      <c r="M28" s="99" t="s">
-        <v>40</v>
-      </c>
-      <c r="N28" s="146"/>
-      <c r="O28" s="146"/>
-      <c r="P28" s="87"/>
-      <c r="Q28" s="74"/>
-      <c r="R28" s="74"/>
-    </row>
-    <row r="29" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="102">
-        <v>1</v>
-      </c>
-      <c r="B29" s="102">
-        <v>2</v>
-      </c>
-      <c r="C29" s="102">
-        <v>3</v>
-      </c>
-      <c r="D29" s="102">
-        <v>4</v>
-      </c>
-      <c r="E29" s="102">
-        <v>5</v>
-      </c>
-      <c r="F29" s="102">
-        <v>6</v>
-      </c>
-      <c r="G29" s="102">
-        <v>7</v>
-      </c>
-      <c r="H29" s="102">
-        <v>8</v>
-      </c>
-      <c r="I29" s="102">
-        <v>9</v>
-      </c>
-      <c r="J29" s="102">
-        <v>10</v>
-      </c>
-      <c r="K29" s="102">
-        <v>11</v>
-      </c>
-      <c r="L29" s="102">
-        <v>12</v>
-      </c>
-      <c r="M29" s="102">
-        <v>13</v>
-      </c>
-      <c r="N29" s="102">
-        <v>14</v>
-      </c>
-      <c r="O29" s="102">
-        <v>15</v>
-      </c>
-      <c r="P29" s="65"/>
-      <c r="Q29" s="89"/>
-      <c r="R29" s="76"/>
-      <c r="S29" s="58" t="s">
-        <v>45</v>
-      </c>
-      <c r="T29" s="60"/>
-      <c r="U29" s="60"/>
     </row>
     <row r="30" spans="1:23" s="5" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="95"/>
-      <c r="B30" s="95"/>
-      <c r="C30" s="95"/>
-      <c r="D30" s="95"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="96"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
-      <c r="J30" s="96"/>
-      <c r="K30" s="96"/>
-      <c r="L30" s="98"/>
-      <c r="M30" s="98"/>
-      <c r="N30" s="97"/>
-      <c r="O30" s="97"/>
-      <c r="P30" s="64"/>
-      <c r="Q30" s="89"/>
-      <c r="R30" s="76"/>
-      <c r="S30" s="59" t="s">
+      <c r="A30" s="88"/>
+      <c r="B30" s="161"/>
+      <c r="C30" s="88"/>
+      <c r="D30" s="88"/>
+      <c r="E30" s="81"/>
+      <c r="F30" s="81"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="88"/>
+      <c r="I30" s="89"/>
+      <c r="J30" s="89"/>
+      <c r="K30" s="89"/>
+      <c r="L30" s="89"/>
+      <c r="M30" s="89"/>
+      <c r="N30" s="89"/>
+      <c r="O30" s="89"/>
+      <c r="P30" s="91"/>
+      <c r="Q30" s="91"/>
+      <c r="R30" s="90"/>
+      <c r="S30" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="T30" s="100" t="s">
+        <v>57</v>
+      </c>
+      <c r="U30" s="162" t="s">
         <v>55</v>
       </c>
-      <c r="T30" s="59" t="s">
-        <v>56</v>
-      </c>
-      <c r="U30" s="61" t="s">
-        <v>57</v>
-      </c>
+      <c r="V30" s="161"/>
+      <c r="W30" s="161"/>
     </row>
     <row r="31" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="76"/>
-      <c r="B31" s="76"/>
-      <c r="C31" s="90"/>
-      <c r="D31" s="90"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="73"/>
-      <c r="G31" s="73"/>
-      <c r="H31" s="73"/>
-      <c r="I31" s="73"/>
-      <c r="J31" s="73"/>
-      <c r="K31" s="73"/>
-      <c r="L31" s="63"/>
-      <c r="M31" s="91"/>
-      <c r="N31" s="69"/>
-      <c r="O31" s="72"/>
-      <c r="P31" s="64"/>
-      <c r="Q31" s="89"/>
-      <c r="R31" s="76"/>
-      <c r="S31" s="59" t="s">
-        <v>58</v>
-      </c>
-      <c r="T31" s="59" t="s">
-        <v>59</v>
-      </c>
-      <c r="U31" s="61" t="s">
-        <v>57</v>
+      <c r="A31" s="73"/>
+      <c r="B31" s="73"/>
+      <c r="C31" s="83"/>
+      <c r="D31" s="83"/>
+      <c r="E31" s="71"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="71"/>
+      <c r="H31" s="71"/>
+      <c r="I31" s="71"/>
+      <c r="J31" s="71"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="62"/>
+      <c r="M31" s="84"/>
+      <c r="N31" s="67"/>
+      <c r="O31" s="70"/>
+      <c r="P31" s="63"/>
+      <c r="Q31" s="49"/>
+      <c r="R31" s="49"/>
+      <c r="S31" s="58">
+        <v>0</v>
+      </c>
+      <c r="T31" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U31" s="60" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B32" s="49"/>
       <c r="C32" s="49"/>
@@ -2362,46 +2377,46 @@
       <c r="P32" s="49"/>
       <c r="Q32" s="49"/>
       <c r="R32" s="49"/>
-      <c r="S32" s="59">
+      <c r="S32" s="58">
         <v>0</v>
       </c>
-      <c r="T32" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U32" s="61" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="33" spans="1:21" s="5" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="156"/>
-      <c r="B33" s="156"/>
-      <c r="C33" s="156"/>
-      <c r="D33" s="156"/>
-      <c r="E33" s="156"/>
-      <c r="F33" s="156"/>
-      <c r="G33" s="155"/>
-      <c r="H33" s="155"/>
-      <c r="I33" s="155"/>
-      <c r="J33" s="155"/>
-      <c r="K33" s="155"/>
-      <c r="L33" s="155"/>
-      <c r="M33" s="155"/>
-      <c r="N33" s="155"/>
-      <c r="O33" s="155"/>
+      <c r="T32" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U32" s="60" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" s="5" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="128"/>
+      <c r="B33" s="128"/>
+      <c r="C33" s="128"/>
+      <c r="D33" s="128"/>
+      <c r="E33" s="128"/>
+      <c r="F33" s="128"/>
+      <c r="G33" s="112"/>
+      <c r="H33" s="112"/>
+      <c r="I33" s="112"/>
+      <c r="J33" s="112"/>
+      <c r="K33" s="112"/>
+      <c r="L33" s="112"/>
+      <c r="M33" s="112"/>
+      <c r="N33" s="112"/>
+      <c r="O33" s="112"/>
       <c r="P33" s="49"/>
-      <c r="Q33" s="49"/>
-      <c r="R33" s="49"/>
-      <c r="S33" s="59">
+      <c r="Q33" s="50"/>
+      <c r="R33" s="50"/>
+      <c r="S33" s="58">
         <v>0</v>
       </c>
-      <c r="T33" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U33" s="61" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T33" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U33" s="60" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15"/>
       <c r="B34" s="50"/>
       <c r="C34" s="50"/>
@@ -2418,236 +2433,281 @@
       <c r="N34" s="50"/>
       <c r="O34" s="50"/>
       <c r="P34" s="50"/>
-      <c r="Q34" s="50"/>
-      <c r="R34" s="50"/>
-      <c r="S34" s="59">
+      <c r="Q34" s="125"/>
+      <c r="R34" s="125"/>
+      <c r="S34" s="58">
         <v>0</v>
       </c>
-      <c r="T34" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U34" s="61" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="35" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="T34" s="58" t="s">
+        <v>55</v>
+      </c>
+      <c r="U34" s="59"/>
+    </row>
+    <row r="35" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="31"/>
       <c r="B35" s="51"/>
       <c r="D35" s="51"/>
       <c r="E35" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="F35" s="157"/>
-      <c r="G35" s="157"/>
-      <c r="H35" s="157"/>
-      <c r="I35" s="67"/>
-      <c r="J35" s="158"/>
-      <c r="K35" s="158"/>
-      <c r="L35" s="158"/>
-      <c r="M35" s="158"/>
-      <c r="N35" s="158"/>
-      <c r="O35" s="158"/>
+        <v>40</v>
+      </c>
+      <c r="F35" s="129"/>
+      <c r="G35" s="129"/>
+      <c r="H35" s="129"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="116"/>
+      <c r="K35" s="116"/>
+      <c r="L35" s="116"/>
+      <c r="M35" s="116"/>
+      <c r="N35" s="116"/>
+      <c r="O35" s="116"/>
       <c r="P35" s="43"/>
-      <c r="Q35" s="138"/>
-      <c r="R35" s="138"/>
-      <c r="S35" s="59">
-        <v>0</v>
-      </c>
-      <c r="T35" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="U35" s="60"/>
-    </row>
-    <row r="36" spans="1:21" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q35" s="125"/>
+      <c r="R35" s="125"/>
+      <c r="S35" s="58"/>
+      <c r="T35" s="58"/>
+      <c r="U35" s="59"/>
+      <c r="V35" s="3"/>
+      <c r="W35" s="3"/>
+    </row>
+    <row r="36" spans="1:23" s="3" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="43"/>
       <c r="B36" s="51"/>
       <c r="C36" s="5"/>
       <c r="D36" s="43"/>
       <c r="E36" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="F36" s="137"/>
-      <c r="G36" s="137"/>
-      <c r="H36" s="137"/>
+        <v>43</v>
+      </c>
+      <c r="F36" s="124"/>
+      <c r="G36" s="124"/>
+      <c r="H36" s="124"/>
       <c r="I36" s="43"/>
-      <c r="J36" s="159"/>
-      <c r="K36" s="159"/>
-      <c r="L36" s="159"/>
-      <c r="M36" s="159"/>
-      <c r="N36" s="159"/>
-      <c r="O36" s="159"/>
+      <c r="J36" s="115"/>
+      <c r="K36" s="115"/>
+      <c r="L36" s="115"/>
+      <c r="M36" s="115"/>
+      <c r="N36" s="115"/>
+      <c r="O36" s="115"/>
       <c r="P36" s="43"/>
-      <c r="Q36" s="138"/>
-      <c r="R36" s="138"/>
-      <c r="S36" s="59"/>
-      <c r="T36" s="59"/>
-      <c r="U36" s="60"/>
-    </row>
-    <row r="37" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="118"/>
-      <c r="B37" s="118"/>
-      <c r="C37" s="118"/>
-      <c r="D37" s="118"/>
+      <c r="Q36" s="131" t="s">
+        <v>42</v>
+      </c>
+      <c r="R36" s="131"/>
+      <c r="S36" s="58"/>
+      <c r="T36" s="58"/>
+      <c r="U36" s="59"/>
+      <c r="V36" s="5"/>
+      <c r="W36" s="5"/>
+    </row>
+    <row r="37" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="130"/>
+      <c r="B37" s="130"/>
+      <c r="C37" s="130"/>
+      <c r="D37" s="130"/>
       <c r="E37" s="4"/>
-      <c r="F37" s="119" t="s">
-        <v>42</v>
-      </c>
-      <c r="G37" s="119"/>
-      <c r="H37" s="119"/>
+      <c r="F37" s="131" t="s">
+        <v>41</v>
+      </c>
+      <c r="G37" s="131"/>
+      <c r="H37" s="131"/>
       <c r="I37" s="33"/>
-      <c r="J37" s="120" t="s">
-        <v>84</v>
-      </c>
-      <c r="K37" s="120"/>
-      <c r="L37" s="120"/>
-      <c r="M37" s="120" t="s">
-        <v>85</v>
-      </c>
-      <c r="N37" s="120"/>
-      <c r="O37" s="120"/>
+      <c r="J37" s="114" t="s">
+        <v>82</v>
+      </c>
+      <c r="K37" s="114"/>
+      <c r="L37" s="114"/>
+      <c r="M37" s="114" t="s">
+        <v>83</v>
+      </c>
+      <c r="N37" s="114"/>
+      <c r="O37" s="114"/>
       <c r="P37" s="33"/>
-      <c r="Q37" s="119" t="s">
-        <v>43</v>
-      </c>
-      <c r="R37" s="119"/>
-      <c r="S37" s="59"/>
-      <c r="T37" s="59"/>
-      <c r="U37" s="60"/>
-    </row>
-    <row r="38" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="90"/>
-      <c r="B38" s="90"/>
-      <c r="C38" s="90"/>
-      <c r="D38" s="90"/>
-      <c r="E38" s="73"/>
-      <c r="F38" s="73"/>
-      <c r="G38" s="73"/>
-      <c r="H38" s="73"/>
-      <c r="I38" s="73"/>
-      <c r="J38" s="73"/>
-      <c r="K38" s="73"/>
-      <c r="L38" s="64"/>
-      <c r="M38" s="66"/>
-      <c r="N38" s="92"/>
-      <c r="O38" s="83"/>
-      <c r="P38" s="93"/>
-      <c r="Q38" s="94"/>
-      <c r="R38" s="76"/>
-      <c r="S38" s="59"/>
-      <c r="T38" s="59"/>
-      <c r="U38" s="60"/>
-    </row>
-    <row r="39" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="S39" s="59"/>
-      <c r="T39" s="59"/>
-      <c r="U39" s="60" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="40" spans="1:21" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:21" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:21" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:21" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:21" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:21" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:21" ht="15" x14ac:dyDescent="0.25">
-      <c r="A48" s="62"/>
-      <c r="B48" s="62"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
-      <c r="K48" s="62"/>
-      <c r="L48" s="62"/>
-      <c r="M48" s="62"/>
-      <c r="N48" s="62"/>
-      <c r="O48" s="62"/>
-      <c r="P48" s="62"/>
-      <c r="Q48" s="62"/>
-      <c r="R48" s="62"/>
+      <c r="Q37" s="87"/>
+      <c r="R37" s="73"/>
+      <c r="S37" s="58"/>
+      <c r="T37" s="58"/>
+      <c r="U37" s="59"/>
+    </row>
+    <row r="38" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="83"/>
+      <c r="B38" s="83"/>
+      <c r="C38" s="83"/>
+      <c r="D38" s="83"/>
+      <c r="E38" s="71"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="71"/>
+      <c r="H38" s="71"/>
+      <c r="I38" s="71"/>
+      <c r="J38" s="71"/>
+      <c r="K38" s="71"/>
+      <c r="L38" s="63"/>
+      <c r="M38" s="64"/>
+      <c r="N38" s="85"/>
+      <c r="O38" s="80"/>
+      <c r="P38" s="86"/>
+      <c r="S38" s="58"/>
+      <c r="T38" s="58"/>
+      <c r="U38" s="59" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q39" s="13"/>
+      <c r="R39" s="13"/>
+      <c r="S39" s="13"/>
+      <c r="T39" s="13"/>
+      <c r="U39" s="13"/>
+      <c r="V39" s="13"/>
+      <c r="W39" s="13"/>
+    </row>
+    <row r="40" spans="1:23" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:23" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q41" s="15"/>
+      <c r="R41" s="15"/>
+      <c r="S41" s="15"/>
+      <c r="T41" s="15"/>
+      <c r="U41" s="15"/>
+      <c r="V41" s="15"/>
+      <c r="W41" s="15"/>
+    </row>
+    <row r="42" spans="1:23" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
+      <c r="S42" s="5"/>
+      <c r="T42" s="5"/>
+      <c r="U42" s="5"/>
+      <c r="V42" s="5"/>
+      <c r="W42" s="5"/>
+    </row>
+    <row r="43" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q43" s="4"/>
+      <c r="R43" s="4"/>
+      <c r="S43" s="4"/>
+      <c r="T43" s="4"/>
+      <c r="U43" s="4"/>
+      <c r="V43" s="4"/>
+      <c r="W43" s="4"/>
+    </row>
+    <row r="44" spans="1:23" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q44" s="16"/>
+      <c r="R44" s="16"/>
+      <c r="S44" s="16"/>
+      <c r="T44" s="16"/>
+      <c r="U44" s="16"/>
+      <c r="V44" s="16"/>
+      <c r="W44" s="16"/>
+    </row>
+    <row r="45" spans="1:23" s="16" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q45" s="5"/>
+      <c r="R45" s="5"/>
+      <c r="S45" s="5"/>
+      <c r="T45" s="5"/>
+      <c r="U45" s="5"/>
+      <c r="V45" s="5"/>
+      <c r="W45" s="5"/>
+    </row>
+    <row r="46" spans="1:23" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
+      <c r="S46" s="4"/>
+      <c r="T46" s="4"/>
+      <c r="U46" s="4"/>
+      <c r="V46" s="4"/>
+      <c r="W46" s="4"/>
+    </row>
+    <row r="47" spans="1:23" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q47" s="61"/>
+      <c r="R47" s="61"/>
+      <c r="S47" s="6"/>
+      <c r="T47" s="6"/>
+      <c r="U47" s="6"/>
+      <c r="V47" s="6"/>
+      <c r="W47" s="6"/>
+    </row>
+    <row r="48" spans="1:23" ht="15" x14ac:dyDescent="0.25">
+      <c r="A48" s="61"/>
+      <c r="B48" s="61"/>
+      <c r="C48" s="61"/>
+      <c r="D48" s="61"/>
+      <c r="E48" s="61"/>
+      <c r="F48" s="61"/>
+      <c r="G48" s="61"/>
+      <c r="H48" s="61"/>
+      <c r="I48" s="61"/>
+      <c r="J48" s="61"/>
+      <c r="K48" s="61"/>
+      <c r="L48" s="61"/>
+      <c r="M48" s="61"/>
+      <c r="N48" s="61"/>
+      <c r="O48" s="61"/>
+      <c r="P48" s="61"/>
+      <c r="Q48" s="61"/>
+      <c r="R48" s="61"/>
     </row>
     <row r="49" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="A49" s="62"/>
-      <c r="B49" s="62"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
-      <c r="E49" s="62"/>
-      <c r="F49" s="62"/>
-      <c r="G49" s="62"/>
-      <c r="H49" s="62"/>
-      <c r="I49" s="62"/>
-      <c r="J49" s="62"/>
-      <c r="K49" s="62"/>
-      <c r="L49" s="62"/>
-      <c r="M49" s="62"/>
-      <c r="N49" s="62"/>
-      <c r="O49" s="62"/>
-      <c r="P49" s="62"/>
-      <c r="Q49" s="62"/>
-      <c r="R49" s="62"/>
+      <c r="A49" s="61"/>
+      <c r="B49" s="61"/>
+      <c r="C49" s="61"/>
+      <c r="D49" s="61"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="61"/>
+      <c r="G49" s="61"/>
+      <c r="H49" s="61"/>
+      <c r="I49" s="61"/>
+      <c r="J49" s="61"/>
+      <c r="K49" s="61"/>
+      <c r="L49" s="61"/>
+      <c r="M49" s="61"/>
+      <c r="N49" s="61"/>
+      <c r="O49" s="61"/>
+      <c r="P49" s="61"/>
+      <c r="Q49" s="61"/>
+      <c r="R49" s="61"/>
     </row>
     <row r="50" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="A50" s="62"/>
-      <c r="B50" s="62"/>
-      <c r="C50" s="62"/>
-      <c r="D50" s="62"/>
-      <c r="E50" s="62"/>
-      <c r="F50" s="62"/>
-      <c r="G50" s="62"/>
-      <c r="H50" s="62"/>
-      <c r="I50" s="62"/>
-      <c r="J50" s="62"/>
-      <c r="K50" s="62"/>
-      <c r="L50" s="62"/>
-      <c r="M50" s="62"/>
-      <c r="N50" s="62"/>
-      <c r="O50" s="62"/>
-      <c r="P50" s="62"/>
-      <c r="Q50" s="62"/>
-      <c r="R50" s="62"/>
+      <c r="A50" s="61"/>
+      <c r="B50" s="61"/>
+      <c r="C50" s="61"/>
+      <c r="D50" s="61"/>
+      <c r="E50" s="61"/>
+      <c r="F50" s="61"/>
+      <c r="G50" s="61"/>
+      <c r="H50" s="61"/>
+      <c r="I50" s="61"/>
+      <c r="J50" s="61"/>
+      <c r="K50" s="61"/>
+      <c r="L50" s="61"/>
+      <c r="M50" s="61"/>
+      <c r="N50" s="61"/>
+      <c r="O50" s="61"/>
+      <c r="P50" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="57">
-    <mergeCell ref="J37:L37"/>
-    <mergeCell ref="M37:O37"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J35:L35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="M36:O36"/>
-    <mergeCell ref="B20:W20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="A27:A28"/>
+  <mergeCells count="59">
+    <mergeCell ref="B20:P20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:G21"/>
     <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="E27:E28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B26:O26"/>
     <mergeCell ref="F27:F28"/>
     <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:M27"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="W21:W22"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="M27:Q27"/>
+    <mergeCell ref="B26:W26"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G14:L14"/>
+    <mergeCell ref="G15:L15"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="L12:O12"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="F37:H37"/>
-    <mergeCell ref="Q37:R37"/>
+    <mergeCell ref="Q36:R36"/>
     <mergeCell ref="G3:I3"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="H5:L5"/>
@@ -2661,16 +2721,27 @@
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="F10:H10"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="L12:O12"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G14:L14"/>
-    <mergeCell ref="G15:L15"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="Q35:R35"/>
+    <mergeCell ref="P21:P22"/>
+    <mergeCell ref="L21:M21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="Q34:R34"/>
+    <mergeCell ref="R27:R28"/>
+    <mergeCell ref="W27:W28"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="J37:L37"/>
+    <mergeCell ref="M37:O37"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="J35:L35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M36:O36"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.31496062992125984" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.11811023622047245"/>
   <pageSetup paperSize="9" scale="83" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Update publish and data
</commit_message>
<xml_diff>
--- a/data/Excel/package_passport.xlsx
+++ b/data/Excel/package_passport.xlsx
@@ -12,11 +12,11 @@
     <workbookView xWindow="930" yWindow="0" windowWidth="22635" windowHeight="9675"/>
   </bookViews>
   <sheets>
-    <sheet name="package_passport" sheetId="1" r:id="rId1"/>
+    <sheet name="Паспорт на упаковку" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="multirow">package_passport!#REF!</definedName>
-    <definedName name="multirow2">package_passport!#REF!</definedName>
+    <definedName name="multirow">'Паспорт на упаковку'!#REF!</definedName>
+    <definedName name="multirow2">'Паспорт на упаковку'!#REF!</definedName>
     <definedName name="S1_Наименование_радионуклида">#REF!</definedName>
   </definedNames>
   <calcPr calcId="152511" fullPrecision="0"/>
@@ -986,8 +986,120 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="26" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -999,131 +1111,19 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="24" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="26" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="26" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1493,14 +1493,14 @@
       <c r="F3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="141"/>
-      <c r="H3" s="142"/>
-      <c r="I3" s="142"/>
+      <c r="G3" s="121"/>
+      <c r="H3" s="122"/>
+      <c r="I3" s="122"/>
       <c r="J3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="143"/>
-      <c r="L3" s="144"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="124"/>
       <c r="M3" s="25"/>
       <c r="N3" s="26"/>
       <c r="O3" s="22"/>
@@ -1545,11 +1545,11 @@
       <c r="G5" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="145"/>
-      <c r="I5" s="146"/>
-      <c r="J5" s="146"/>
-      <c r="K5" s="146"/>
-      <c r="L5" s="146"/>
+      <c r="H5" s="125"/>
+      <c r="I5" s="126"/>
+      <c r="J5" s="126"/>
+      <c r="K5" s="126"/>
+      <c r="L5" s="126"/>
       <c r="M5" s="31"/>
       <c r="N5" s="31"/>
       <c r="O5" s="31"/>
@@ -1568,13 +1568,13 @@
       <c r="E6" s="33"/>
       <c r="F6" s="33"/>
       <c r="G6" s="33"/>
-      <c r="H6" s="147" t="s">
+      <c r="H6" s="113" t="s">
         <v>5</v>
       </c>
-      <c r="I6" s="148"/>
-      <c r="J6" s="148"/>
-      <c r="K6" s="148"/>
-      <c r="L6" s="148"/>
+      <c r="I6" s="127"/>
+      <c r="J6" s="127"/>
+      <c r="K6" s="127"/>
+      <c r="L6" s="127"/>
       <c r="M6" s="33"/>
       <c r="N6" s="33"/>
       <c r="O6" s="33"/>
@@ -1589,11 +1589,11 @@
       <c r="G7" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="152"/>
-      <c r="I7" s="152"/>
-      <c r="J7" s="152"/>
-      <c r="K7" s="152"/>
-      <c r="L7" s="152"/>
+      <c r="H7" s="131"/>
+      <c r="I7" s="131"/>
+      <c r="J7" s="131"/>
+      <c r="K7" s="131"/>
+      <c r="L7" s="131"/>
       <c r="S7" s="55">
         <v>4</v>
       </c>
@@ -1608,19 +1608,19 @@
       <c r="B9" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="149"/>
-      <c r="D9" s="150"/>
+      <c r="C9" s="128"/>
+      <c r="D9" s="129"/>
       <c r="E9" s="31"/>
-      <c r="F9" s="145"/>
-      <c r="G9" s="145"/>
-      <c r="H9" s="145"/>
+      <c r="F9" s="125"/>
+      <c r="G9" s="125"/>
+      <c r="H9" s="125"/>
       <c r="I9" s="34"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
-      <c r="L9" s="153"/>
-      <c r="M9" s="153"/>
-      <c r="N9" s="153"/>
-      <c r="O9" s="153"/>
+      <c r="L9" s="132"/>
+      <c r="M9" s="132"/>
+      <c r="N9" s="132"/>
+      <c r="O9" s="132"/>
       <c r="P9" s="34"/>
       <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
@@ -1641,22 +1641,22 @@
       <c r="C10" s="52"/>
       <c r="D10" s="35"/>
       <c r="E10" s="35"/>
-      <c r="F10" s="147" t="s">
+      <c r="F10" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="G10" s="147"/>
-      <c r="H10" s="147"/>
+      <c r="G10" s="113"/>
+      <c r="H10" s="113"/>
       <c r="I10" s="35"/>
       <c r="J10" s="35"/>
       <c r="K10" s="35"/>
-      <c r="L10" s="147" t="s">
+      <c r="L10" s="113" t="s">
         <v>69</v>
       </c>
-      <c r="M10" s="147"/>
-      <c r="N10" s="147" t="s">
+      <c r="M10" s="113"/>
+      <c r="N10" s="113" t="s">
         <v>68</v>
       </c>
-      <c r="O10" s="147"/>
+      <c r="O10" s="113"/>
       <c r="P10" s="35"/>
       <c r="Q10" s="35"/>
       <c r="R10" s="35"/>
@@ -1671,12 +1671,12 @@
       <c r="F11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="157"/>
-      <c r="H11" s="157"/>
+      <c r="G11" s="115"/>
+      <c r="H11" s="115"/>
       <c r="I11" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="J11" s="113"/>
+      <c r="J11" s="149"/>
       <c r="K11" s="39"/>
       <c r="L11" s="31"/>
       <c r="M11" s="31"/>
@@ -1696,15 +1696,15 @@
       <c r="F12" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="155"/>
-      <c r="H12" s="155"/>
-      <c r="I12" s="155"/>
+      <c r="G12" s="116"/>
+      <c r="H12" s="116"/>
+      <c r="I12" s="116"/>
       <c r="J12" s="39"/>
       <c r="K12" s="31"/>
-      <c r="L12" s="156"/>
-      <c r="M12" s="156"/>
-      <c r="N12" s="156"/>
-      <c r="O12" s="156"/>
+      <c r="L12" s="117"/>
+      <c r="M12" s="117"/>
+      <c r="N12" s="117"/>
+      <c r="O12" s="117"/>
       <c r="P12" s="37"/>
       <c r="Q12" s="31"/>
       <c r="R12" s="31"/>
@@ -1723,12 +1723,12 @@
       <c r="I13" s="45"/>
       <c r="J13" s="39"/>
       <c r="K13" s="31"/>
-      <c r="L13" s="147" t="s">
+      <c r="L13" s="113" t="s">
         <v>10</v>
       </c>
-      <c r="M13" s="147"/>
-      <c r="N13" s="147"/>
-      <c r="O13" s="147"/>
+      <c r="M13" s="113"/>
+      <c r="N13" s="113"/>
+      <c r="O13" s="113"/>
       <c r="P13" s="37"/>
       <c r="Q13" s="41"/>
       <c r="R13" s="28"/>
@@ -1742,17 +1742,17 @@
       <c r="F14" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="G14" s="156"/>
-      <c r="H14" s="156"/>
-      <c r="I14" s="156"/>
-      <c r="J14" s="156"/>
-      <c r="K14" s="156"/>
-      <c r="L14" s="156"/>
+      <c r="G14" s="117"/>
+      <c r="H14" s="117"/>
+      <c r="I14" s="117"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="117"/>
+      <c r="L14" s="117"/>
       <c r="M14" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="N14" s="159"/>
-      <c r="O14" s="159"/>
+      <c r="N14" s="150"/>
+      <c r="O14" s="150"/>
       <c r="P14" s="56"/>
       <c r="Q14" s="56"/>
       <c r="R14" s="44"/>
@@ -1766,17 +1766,17 @@
       <c r="F15" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="158"/>
-      <c r="H15" s="158"/>
-      <c r="I15" s="158"/>
-      <c r="J15" s="158"/>
-      <c r="K15" s="158"/>
-      <c r="L15" s="158"/>
+      <c r="G15" s="133"/>
+      <c r="H15" s="133"/>
+      <c r="I15" s="133"/>
+      <c r="J15" s="133"/>
+      <c r="K15" s="133"/>
+      <c r="L15" s="133"/>
       <c r="M15" s="56" t="s">
         <v>82</v>
       </c>
-      <c r="N15" s="160"/>
-      <c r="O15" s="160"/>
+      <c r="N15" s="151"/>
+      <c r="O15" s="151"/>
       <c r="P15" s="56"/>
       <c r="Q15" s="57"/>
       <c r="R15" s="57"/>
@@ -1790,17 +1790,17 @@
       <c r="F16" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="145"/>
-      <c r="H16" s="145"/>
-      <c r="I16" s="145"/>
+      <c r="G16" s="125"/>
+      <c r="H16" s="125"/>
+      <c r="I16" s="125"/>
       <c r="J16" s="39"/>
       <c r="K16" s="31"/>
       <c r="L16" s="31"/>
       <c r="M16" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="N16" s="154"/>
-      <c r="O16" s="154"/>
+      <c r="N16" s="114"/>
+      <c r="O16" s="114"/>
       <c r="P16" s="31"/>
       <c r="Q16" s="45"/>
       <c r="R16" s="31"/>
@@ -1814,11 +1814,11 @@
       <c r="F17" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="114"/>
-      <c r="H17" s="115" t="s">
+      <c r="G17" s="152"/>
+      <c r="H17" s="153" t="s">
         <v>83</v>
       </c>
-      <c r="I17" s="116"/>
+      <c r="I17" s="154"/>
       <c r="J17" s="45"/>
       <c r="K17" s="43"/>
       <c r="L17" s="43"/>
@@ -1838,7 +1838,7 @@
       <c r="F18" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="G18" s="118"/>
+      <c r="G18" s="160"/>
       <c r="H18" s="45"/>
       <c r="I18" s="45"/>
       <c r="J18" s="45"/>
@@ -1847,8 +1847,8 @@
       <c r="M18" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="N18" s="151"/>
-      <c r="O18" s="151"/>
+      <c r="N18" s="130"/>
+      <c r="O18" s="130"/>
       <c r="P18" s="43"/>
       <c r="Q18" s="45"/>
       <c r="R18" s="37"/>
@@ -1880,67 +1880,67 @@
       <c r="A20" s="103" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="122" t="s">
+      <c r="B20" s="143" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="123"/>
-      <c r="D20" s="123"/>
-      <c r="E20" s="123"/>
-      <c r="F20" s="123"/>
-      <c r="G20" s="123"/>
-      <c r="H20" s="123"/>
-      <c r="I20" s="123"/>
-      <c r="J20" s="123"/>
-      <c r="K20" s="123"/>
-      <c r="L20" s="123"/>
-      <c r="M20" s="123"/>
-      <c r="N20" s="123"/>
-      <c r="O20" s="123"/>
-      <c r="P20" s="123"/>
-      <c r="Q20" s="123"/>
-      <c r="R20" s="123"/>
-      <c r="S20" s="123"/>
-      <c r="T20" s="123"/>
-      <c r="U20" s="123"/>
-      <c r="V20" s="123"/>
-      <c r="W20" s="124"/>
+      <c r="C20" s="144"/>
+      <c r="D20" s="144"/>
+      <c r="E20" s="144"/>
+      <c r="F20" s="144"/>
+      <c r="G20" s="144"/>
+      <c r="H20" s="144"/>
+      <c r="I20" s="144"/>
+      <c r="J20" s="144"/>
+      <c r="K20" s="144"/>
+      <c r="L20" s="144"/>
+      <c r="M20" s="144"/>
+      <c r="N20" s="144"/>
+      <c r="O20" s="144"/>
+      <c r="P20" s="144"/>
+      <c r="Q20" s="144"/>
+      <c r="R20" s="144"/>
+      <c r="S20" s="144"/>
+      <c r="T20" s="144"/>
+      <c r="U20" s="144"/>
+      <c r="V20" s="144"/>
+      <c r="W20" s="145"/>
     </row>
     <row r="21" spans="1:23" s="7" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="127" t="s">
+      <c r="A21" s="134" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="128"/>
-      <c r="C21" s="128"/>
-      <c r="D21" s="128"/>
-      <c r="E21" s="128"/>
-      <c r="F21" s="129"/>
-      <c r="G21" s="127" t="s">
+      <c r="B21" s="135"/>
+      <c r="C21" s="135"/>
+      <c r="D21" s="135"/>
+      <c r="E21" s="135"/>
+      <c r="F21" s="136"/>
+      <c r="G21" s="134" t="s">
         <v>20</v>
       </c>
-      <c r="H21" s="128"/>
-      <c r="I21" s="128"/>
-      <c r="J21" s="129"/>
-      <c r="K21" s="125" t="s">
+      <c r="H21" s="135"/>
+      <c r="I21" s="135"/>
+      <c r="J21" s="136"/>
+      <c r="K21" s="141" t="s">
         <v>80</v>
       </c>
-      <c r="L21" s="126"/>
-      <c r="M21" s="125" t="s">
+      <c r="L21" s="142"/>
+      <c r="M21" s="141" t="s">
         <v>81</v>
       </c>
-      <c r="N21" s="126"/>
-      <c r="O21" s="125" t="s">
+      <c r="N21" s="142"/>
+      <c r="O21" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="P21" s="126"/>
-      <c r="Q21" s="125" t="s">
+      <c r="P21" s="142"/>
+      <c r="Q21" s="141" t="s">
         <v>62</v>
       </c>
-      <c r="R21" s="126"/>
+      <c r="R21" s="142"/>
       <c r="S21" s="70"/>
       <c r="T21" s="112"/>
       <c r="U21" s="112"/>
       <c r="V21" s="112"/>
-      <c r="W21" s="135" t="s">
+      <c r="W21" s="139" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       <c r="T22" s="105"/>
       <c r="U22" s="105"/>
       <c r="V22" s="112"/>
-      <c r="W22" s="136"/>
+      <c r="W22" s="140"/>
     </row>
     <row r="23" spans="1:23" s="8" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="100">
@@ -2126,22 +2126,22 @@
       <c r="A26" s="103" t="s">
         <v>51</v>
       </c>
-      <c r="B26" s="132" t="s">
+      <c r="B26" s="148" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="132"/>
-      <c r="D26" s="132"/>
-      <c r="E26" s="132"/>
-      <c r="F26" s="132"/>
-      <c r="G26" s="132"/>
-      <c r="H26" s="132"/>
-      <c r="I26" s="132"/>
-      <c r="J26" s="132"/>
-      <c r="K26" s="132"/>
-      <c r="L26" s="132"/>
-      <c r="M26" s="132"/>
-      <c r="N26" s="132"/>
-      <c r="O26" s="132"/>
+      <c r="C26" s="148"/>
+      <c r="D26" s="148"/>
+      <c r="E26" s="148"/>
+      <c r="F26" s="148"/>
+      <c r="G26" s="148"/>
+      <c r="H26" s="148"/>
+      <c r="I26" s="148"/>
+      <c r="J26" s="148"/>
+      <c r="K26" s="148"/>
+      <c r="L26" s="148"/>
+      <c r="M26" s="148"/>
+      <c r="N26" s="148"/>
+      <c r="O26" s="148"/>
       <c r="P26" s="86"/>
       <c r="Q26" s="86"/>
       <c r="R26" s="86"/>
@@ -2152,41 +2152,41 @@
       <c r="W26" s="82"/>
     </row>
     <row r="27" spans="1:23" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="130" t="s">
+      <c r="A27" s="146" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="130" t="s">
+      <c r="B27" s="146" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="130" t="s">
+      <c r="C27" s="146" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="131" t="s">
+      <c r="D27" s="147" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="130" t="s">
+      <c r="E27" s="146" t="s">
         <v>81</v>
       </c>
-      <c r="F27" s="130" t="s">
+      <c r="F27" s="146" t="s">
         <v>30</v>
       </c>
-      <c r="G27" s="130" t="s">
+      <c r="G27" s="146" t="s">
         <v>34</v>
       </c>
-      <c r="H27" s="130" t="s">
+      <c r="H27" s="146" t="s">
         <v>35</v>
       </c>
-      <c r="I27" s="130" t="s">
+      <c r="I27" s="146" t="s">
         <v>79</v>
       </c>
-      <c r="J27" s="130"/>
-      <c r="K27" s="130"/>
-      <c r="L27" s="130"/>
-      <c r="M27" s="130"/>
-      <c r="N27" s="130" t="s">
+      <c r="J27" s="146"/>
+      <c r="K27" s="146"/>
+      <c r="L27" s="146"/>
+      <c r="M27" s="146"/>
+      <c r="N27" s="146" t="s">
         <v>36</v>
       </c>
-      <c r="O27" s="130" t="s">
+      <c r="O27" s="146" t="s">
         <v>78</v>
       </c>
       <c r="P27" s="87"/>
@@ -2199,14 +2199,14 @@
       <c r="W27" s="84"/>
     </row>
     <row r="28" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="130"/>
-      <c r="B28" s="130"/>
-      <c r="C28" s="130"/>
-      <c r="D28" s="131"/>
-      <c r="E28" s="130"/>
-      <c r="F28" s="130"/>
-      <c r="G28" s="130"/>
-      <c r="H28" s="130"/>
+      <c r="A28" s="146"/>
+      <c r="B28" s="146"/>
+      <c r="C28" s="146"/>
+      <c r="D28" s="147"/>
+      <c r="E28" s="146"/>
+      <c r="F28" s="146"/>
+      <c r="G28" s="146"/>
+      <c r="H28" s="146"/>
       <c r="I28" s="99" t="s">
         <v>37</v>
       </c>
@@ -2222,8 +2222,8 @@
       <c r="M28" s="99" t="s">
         <v>40</v>
       </c>
-      <c r="N28" s="130"/>
-      <c r="O28" s="130"/>
+      <c r="N28" s="146"/>
+      <c r="O28" s="146"/>
       <c r="P28" s="87"/>
       <c r="Q28" s="74"/>
       <c r="R28" s="74"/>
@@ -2373,21 +2373,21 @@
       </c>
     </row>
     <row r="33" spans="1:21" s="5" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="137"/>
-      <c r="B33" s="137"/>
-      <c r="C33" s="137"/>
-      <c r="D33" s="137"/>
-      <c r="E33" s="137"/>
-      <c r="F33" s="137"/>
-      <c r="G33" s="117"/>
-      <c r="H33" s="117"/>
-      <c r="I33" s="117"/>
-      <c r="J33" s="117"/>
-      <c r="K33" s="117"/>
-      <c r="L33" s="117"/>
-      <c r="M33" s="117"/>
-      <c r="N33" s="117"/>
-      <c r="O33" s="117"/>
+      <c r="A33" s="156"/>
+      <c r="B33" s="156"/>
+      <c r="C33" s="156"/>
+      <c r="D33" s="156"/>
+      <c r="E33" s="156"/>
+      <c r="F33" s="156"/>
+      <c r="G33" s="155"/>
+      <c r="H33" s="155"/>
+      <c r="I33" s="155"/>
+      <c r="J33" s="155"/>
+      <c r="K33" s="155"/>
+      <c r="L33" s="155"/>
+      <c r="M33" s="155"/>
+      <c r="N33" s="155"/>
+      <c r="O33" s="155"/>
       <c r="P33" s="49"/>
       <c r="Q33" s="49"/>
       <c r="R33" s="49"/>
@@ -2437,19 +2437,19 @@
       <c r="E35" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="F35" s="138"/>
-      <c r="G35" s="138"/>
-      <c r="H35" s="138"/>
+      <c r="F35" s="157"/>
+      <c r="G35" s="157"/>
+      <c r="H35" s="157"/>
       <c r="I35" s="67"/>
-      <c r="J35" s="121"/>
-      <c r="K35" s="121"/>
-      <c r="L35" s="121"/>
-      <c r="M35" s="121"/>
-      <c r="N35" s="121"/>
-      <c r="O35" s="121"/>
+      <c r="J35" s="158"/>
+      <c r="K35" s="158"/>
+      <c r="L35" s="158"/>
+      <c r="M35" s="158"/>
+      <c r="N35" s="158"/>
+      <c r="O35" s="158"/>
       <c r="P35" s="43"/>
-      <c r="Q35" s="134"/>
-      <c r="R35" s="134"/>
+      <c r="Q35" s="138"/>
+      <c r="R35" s="138"/>
       <c r="S35" s="59">
         <v>0</v>
       </c>
@@ -2466,50 +2466,50 @@
       <c r="E36" s="36" t="s">
         <v>44</v>
       </c>
-      <c r="F36" s="133"/>
-      <c r="G36" s="133"/>
-      <c r="H36" s="133"/>
+      <c r="F36" s="137"/>
+      <c r="G36" s="137"/>
+      <c r="H36" s="137"/>
       <c r="I36" s="43"/>
-      <c r="J36" s="120"/>
-      <c r="K36" s="120"/>
-      <c r="L36" s="120"/>
-      <c r="M36" s="120"/>
-      <c r="N36" s="120"/>
-      <c r="O36" s="120"/>
+      <c r="J36" s="159"/>
+      <c r="K36" s="159"/>
+      <c r="L36" s="159"/>
+      <c r="M36" s="159"/>
+      <c r="N36" s="159"/>
+      <c r="O36" s="159"/>
       <c r="P36" s="43"/>
-      <c r="Q36" s="134"/>
-      <c r="R36" s="134"/>
+      <c r="Q36" s="138"/>
+      <c r="R36" s="138"/>
       <c r="S36" s="59"/>
       <c r="T36" s="59"/>
       <c r="U36" s="60"/>
     </row>
     <row r="37" spans="1:21" s="5" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="139"/>
-      <c r="B37" s="139"/>
-      <c r="C37" s="139"/>
-      <c r="D37" s="139"/>
+      <c r="A37" s="118"/>
+      <c r="B37" s="118"/>
+      <c r="C37" s="118"/>
+      <c r="D37" s="118"/>
       <c r="E37" s="4"/>
-      <c r="F37" s="140" t="s">
+      <c r="F37" s="119" t="s">
         <v>42</v>
       </c>
-      <c r="G37" s="140"/>
-      <c r="H37" s="140"/>
+      <c r="G37" s="119"/>
+      <c r="H37" s="119"/>
       <c r="I37" s="33"/>
-      <c r="J37" s="119" t="s">
+      <c r="J37" s="120" t="s">
         <v>84</v>
       </c>
-      <c r="K37" s="119"/>
-      <c r="L37" s="119"/>
-      <c r="M37" s="119" t="s">
+      <c r="K37" s="120"/>
+      <c r="L37" s="120"/>
+      <c r="M37" s="120" t="s">
         <v>85</v>
       </c>
-      <c r="N37" s="119"/>
-      <c r="O37" s="119"/>
+      <c r="N37" s="120"/>
+      <c r="O37" s="120"/>
       <c r="P37" s="33"/>
-      <c r="Q37" s="140" t="s">
+      <c r="Q37" s="119" t="s">
         <v>43</v>
       </c>
-      <c r="R37" s="140"/>
+      <c r="R37" s="119"/>
       <c r="S37" s="59"/>
       <c r="T37" s="59"/>
       <c r="U37" s="60"/>
@@ -2614,16 +2614,37 @@
     </row>
   </sheetData>
   <mergeCells count="57">
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G14:L14"/>
-    <mergeCell ref="G15:L15"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="J37:L37"/>
+    <mergeCell ref="M37:O37"/>
+    <mergeCell ref="J36:L36"/>
+    <mergeCell ref="J35:L35"/>
+    <mergeCell ref="M35:O35"/>
+    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="B20:W20"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="B26:O26"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="I27:M27"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="F36:H36"/>
+    <mergeCell ref="Q36:R36"/>
+    <mergeCell ref="W21:W22"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="Q35:R35"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="F37:H37"/>
     <mergeCell ref="Q37:R37"/>
@@ -2640,37 +2661,16 @@
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="F10:H10"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="W21:W22"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="Q35:R35"/>
-    <mergeCell ref="B20:W20"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="B26:O26"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:H28"/>
-    <mergeCell ref="I27:M27"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="J37:L37"/>
-    <mergeCell ref="M37:O37"/>
-    <mergeCell ref="J36:L36"/>
-    <mergeCell ref="J35:L35"/>
-    <mergeCell ref="M35:O35"/>
-    <mergeCell ref="M36:O36"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="L12:O12"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G14:L14"/>
+    <mergeCell ref="G15:L15"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="N15:O15"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.31496062992125984" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.11811023622047245"/>
   <pageSetup paperSize="9" scale="83" orientation="landscape" r:id="rId1"/>

</xml_diff>